<commit_message>
Update MLB hitter fantasy scores 2026-08-10 (2026-08-09 09:04 PM)
</commit_message>
<xml_diff>
--- a/PRIZEPICKS_HITTER_AI_V5_TOP30_2026_08_10.xlsx
+++ b/PRIZEPICKS_HITTER_AI_V5_TOP30_2026_08_10.xlsx
@@ -2145,7 +2145,7 @@
         <v>7.09</v>
       </c>
       <c r="R2" s="3" t="n">
-        <v>0.736</v>
+        <v>0.737</v>
       </c>
       <c r="S2" s="3" t="n">
         <v>6.4</v>
@@ -2184,13 +2184,13 @@
         <v>88.8</v>
       </c>
       <c r="AC2" s="5" t="n">
-        <v>83.09999999999999</v>
+        <v>83.2</v>
       </c>
       <c r="AD2" s="5" t="n">
-        <v>82.09999999999999</v>
+        <v>82.2</v>
       </c>
       <c r="AE2" s="5" t="n">
-        <v>77.09999999999999</v>
+        <v>77.2</v>
       </c>
       <c r="AF2" s="5" t="n">
         <v>72.5</v>
@@ -2199,16 +2199,16 @@
         <v>72</v>
       </c>
       <c r="AH2" s="5" t="n">
-        <v>64.59999999999999</v>
+        <v>64.7</v>
       </c>
       <c r="AI2" s="5" t="n">
         <v>61.1</v>
       </c>
       <c r="AJ2" s="6" t="n">
-        <v>53.4</v>
+        <v>53.5</v>
       </c>
       <c r="AK2" s="7" t="n">
-        <v>52.4</v>
+        <v>52.5</v>
       </c>
       <c r="AL2" s="7" t="n">
         <v>49</v>
@@ -2220,7 +2220,7 @@
         <v>45.1</v>
       </c>
       <c r="AO2" s="7" t="n">
-        <v>41.4</v>
+        <v>41.5</v>
       </c>
       <c r="AP2" s="8" t="n">
         <v>38.8</v>
@@ -2232,10 +2232,10 @@
         <v>36</v>
       </c>
       <c r="AS2" s="8" t="n">
-        <v>34.4</v>
+        <v>34.5</v>
       </c>
       <c r="AT2" s="8" t="n">
-        <v>34.4</v>
+        <v>34.5</v>
       </c>
       <c r="AU2" s="8" t="n">
         <v>30.8</v>
@@ -2253,7 +2253,7 @@
         <v>23.8</v>
       </c>
       <c r="AZ2" s="3" t="n">
-        <v>261.89</v>
+        <v>261.9</v>
       </c>
       <c r="BA2" s="4" t="inlineStr">
         <is>
@@ -2745,7 +2745,7 @@
         <v>5.04</v>
       </c>
       <c r="GT2" s="3" t="n">
-        <v>15.34</v>
+        <v>15.35</v>
       </c>
       <c r="GU2" s="3" t="n">
         <v>20.5</v>
@@ -2774,13 +2774,13 @@
         <v>82.8</v>
       </c>
       <c r="HC2" s="3" t="n">
-        <v>77.09999999999999</v>
+        <v>77.2</v>
       </c>
       <c r="HD2" s="3" t="n">
-        <v>77.09999999999999</v>
+        <v>77.2</v>
       </c>
       <c r="HE2" s="3" t="n">
-        <v>72.59999999999999</v>
+        <v>72.7</v>
       </c>
       <c r="HF2" s="3" t="n">
         <v>68.5</v>
@@ -2789,16 +2789,16 @@
         <v>68.5</v>
       </c>
       <c r="HH2" s="3" t="n">
-        <v>61.6</v>
+        <v>61.7</v>
       </c>
       <c r="HI2" s="3" t="n">
         <v>58.6</v>
       </c>
       <c r="HJ2" s="3" t="n">
-        <v>52.4</v>
+        <v>52.5</v>
       </c>
       <c r="HK2" s="3" t="n">
-        <v>52.4</v>
+        <v>52.5</v>
       </c>
       <c r="HL2" s="3" t="n">
         <v>49</v>
@@ -2810,7 +2810,7 @@
         <v>45.1</v>
       </c>
       <c r="HO2" s="3" t="n">
-        <v>41.4</v>
+        <v>41.5</v>
       </c>
       <c r="HP2" s="3" t="n">
         <v>38.8</v>
@@ -2822,10 +2822,10 @@
         <v>36</v>
       </c>
       <c r="HS2" s="3" t="n">
-        <v>34.4</v>
+        <v>34.5</v>
       </c>
       <c r="HT2" s="3" t="n">
-        <v>34.4</v>
+        <v>34.5</v>
       </c>
       <c r="HU2" s="3" t="n">
         <v>30.8</v>
@@ -3826,10 +3826,10 @@
         <v>10.55</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>9.279999999999999</v>
+        <v>9.31</v>
       </c>
       <c r="L4" s="3" t="n">
-        <v>9.279999999999999</v>
+        <v>9.31</v>
       </c>
       <c r="M4" s="3" t="n">
         <v>7.06</v>
@@ -3841,13 +3841,13 @@
         <v>8.029999999999999</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>8.24</v>
+        <v>8.25</v>
       </c>
       <c r="Q4" s="3" t="n">
         <v>8.029999999999999</v>
       </c>
       <c r="R4" s="3" t="n">
-        <v>0.974</v>
+        <v>0.973</v>
       </c>
       <c r="S4" s="3" t="n">
         <v>9</v>
@@ -3874,88 +3874,88 @@
         </is>
       </c>
       <c r="Y4" s="5" t="n">
-        <v>87.2</v>
+        <v>87.3</v>
       </c>
       <c r="Z4" s="5" t="n">
-        <v>87.2</v>
+        <v>87.3</v>
       </c>
       <c r="AA4" s="5" t="n">
-        <v>78</v>
+        <v>78.2</v>
       </c>
       <c r="AB4" s="5" t="n">
-        <v>77.5</v>
+        <v>77.7</v>
       </c>
       <c r="AC4" s="5" t="n">
-        <v>72.8</v>
+        <v>73</v>
       </c>
       <c r="AD4" s="5" t="n">
-        <v>71.8</v>
+        <v>72</v>
       </c>
       <c r="AE4" s="5" t="n">
-        <v>61.6</v>
+        <v>61.7</v>
       </c>
       <c r="AF4" s="5" t="n">
-        <v>61.1</v>
+        <v>61.2</v>
       </c>
       <c r="AG4" s="6" t="n">
-        <v>57.3</v>
+        <v>57.4</v>
       </c>
       <c r="AH4" s="7" t="n">
-        <v>56.8</v>
+        <v>56.9</v>
       </c>
       <c r="AI4" s="7" t="n">
-        <v>49.3</v>
+        <v>49.4</v>
       </c>
       <c r="AJ4" s="7" t="n">
-        <v>47.8</v>
+        <v>47.9</v>
       </c>
       <c r="AK4" s="7" t="n">
-        <v>42.2</v>
+        <v>42.4</v>
       </c>
       <c r="AL4" s="7" t="n">
-        <v>42.2</v>
+        <v>42.4</v>
       </c>
       <c r="AM4" s="8" t="n">
-        <v>38.2</v>
+        <v>38.4</v>
       </c>
       <c r="AN4" s="8" t="n">
-        <v>34.4</v>
+        <v>34.5</v>
       </c>
       <c r="AO4" s="8" t="n">
-        <v>34.4</v>
+        <v>34.5</v>
       </c>
       <c r="AP4" s="8" t="n">
-        <v>32.2</v>
+        <v>32.3</v>
       </c>
       <c r="AQ4" s="8" t="n">
-        <v>32.2</v>
+        <v>32.3</v>
       </c>
       <c r="AR4" s="8" t="n">
-        <v>29.3</v>
+        <v>29.4</v>
       </c>
       <c r="AS4" s="8" t="n">
-        <v>29.3</v>
+        <v>29.4</v>
       </c>
       <c r="AT4" s="8" t="n">
-        <v>27.5</v>
+        <v>27.7</v>
       </c>
       <c r="AU4" s="8" t="n">
-        <v>27.5</v>
+        <v>27.7</v>
       </c>
       <c r="AV4" s="8" t="n">
-        <v>23.2</v>
+        <v>23.3</v>
       </c>
       <c r="AW4" s="8" t="n">
-        <v>23.2</v>
+        <v>23.3</v>
       </c>
       <c r="AX4" s="8" t="n">
-        <v>21.9</v>
+        <v>22</v>
       </c>
       <c r="AY4" s="8" t="n">
-        <v>21.9</v>
+        <v>22</v>
       </c>
       <c r="AZ4" s="3" t="n">
-        <v>238.36</v>
+        <v>238.82</v>
       </c>
       <c r="BA4" s="4" t="inlineStr">
         <is>
@@ -3964,7 +3964,7 @@
       </c>
       <c r="BB4" s="9" t="inlineStr">
         <is>
-          <t>MORE 6.0 | 61.1% | Edge +3.3</t>
+          <t>MORE 6.0 | 61.2% | Edge +3.3</t>
         </is>
       </c>
       <c r="BC4" s="4" t="inlineStr">
@@ -3976,13 +3976,13 @@
         <v>6</v>
       </c>
       <c r="BE4" s="3" t="n">
-        <v>61.1</v>
+        <v>61.2</v>
       </c>
       <c r="BF4" s="3" t="n">
-        <v>3.28</v>
+        <v>3.31</v>
       </c>
       <c r="BG4" s="3" t="n">
-        <v>22.2</v>
+        <v>22.4</v>
       </c>
       <c r="BH4" s="4" t="inlineStr">
         <is>
@@ -4436,13 +4436,13 @@
         <v>8.029999999999999</v>
       </c>
       <c r="GS4" s="3" t="n">
-        <v>3.16</v>
+        <v>3.17</v>
       </c>
       <c r="GT4" s="3" t="n">
-        <v>13.88</v>
+        <v>13.87</v>
       </c>
       <c r="GU4" s="3" t="n">
-        <v>20.7</v>
+        <v>20.68</v>
       </c>
       <c r="GV4" s="3" t="n">
         <v>4.53</v>
@@ -4456,85 +4456,85 @@
         </is>
       </c>
       <c r="GY4" s="3" t="n">
-        <v>79.2</v>
+        <v>79.3</v>
       </c>
       <c r="GZ4" s="3" t="n">
-        <v>79.2</v>
+        <v>79.3</v>
       </c>
       <c r="HA4" s="3" t="n">
-        <v>70.5</v>
+        <v>70.7</v>
       </c>
       <c r="HB4" s="3" t="n">
-        <v>70.5</v>
+        <v>70.7</v>
       </c>
       <c r="HC4" s="3" t="n">
-        <v>66.8</v>
+        <v>67</v>
       </c>
       <c r="HD4" s="3" t="n">
-        <v>66.8</v>
+        <v>67</v>
       </c>
       <c r="HE4" s="3" t="n">
-        <v>57.1</v>
+        <v>57.2</v>
       </c>
       <c r="HF4" s="3" t="n">
-        <v>57.1</v>
+        <v>57.2</v>
       </c>
       <c r="HG4" s="3" t="n">
-        <v>53.8</v>
+        <v>53.9</v>
       </c>
       <c r="HH4" s="3" t="n">
-        <v>53.8</v>
+        <v>53.9</v>
       </c>
       <c r="HI4" s="3" t="n">
-        <v>46.8</v>
+        <v>46.9</v>
       </c>
       <c r="HJ4" s="3" t="n">
-        <v>46.8</v>
+        <v>46.9</v>
       </c>
       <c r="HK4" s="3" t="n">
-        <v>42.2</v>
+        <v>42.4</v>
       </c>
       <c r="HL4" s="3" t="n">
-        <v>42.2</v>
+        <v>42.4</v>
       </c>
       <c r="HM4" s="3" t="n">
-        <v>38.2</v>
+        <v>38.4</v>
       </c>
       <c r="HN4" s="3" t="n">
-        <v>34.4</v>
+        <v>34.5</v>
       </c>
       <c r="HO4" s="3" t="n">
-        <v>34.4</v>
+        <v>34.5</v>
       </c>
       <c r="HP4" s="3" t="n">
-        <v>32.2</v>
+        <v>32.3</v>
       </c>
       <c r="HQ4" s="3" t="n">
-        <v>32.2</v>
+        <v>32.3</v>
       </c>
       <c r="HR4" s="3" t="n">
-        <v>29.3</v>
+        <v>29.4</v>
       </c>
       <c r="HS4" s="3" t="n">
-        <v>29.3</v>
+        <v>29.4</v>
       </c>
       <c r="HT4" s="3" t="n">
-        <v>27.5</v>
+        <v>27.7</v>
       </c>
       <c r="HU4" s="3" t="n">
-        <v>27.5</v>
+        <v>27.7</v>
       </c>
       <c r="HV4" s="3" t="n">
-        <v>23.2</v>
+        <v>23.3</v>
       </c>
       <c r="HW4" s="3" t="n">
-        <v>23.2</v>
+        <v>23.3</v>
       </c>
       <c r="HX4" s="3" t="n">
-        <v>21.9</v>
+        <v>22</v>
       </c>
       <c r="HY4" s="3" t="n">
-        <v>21.9</v>
+        <v>22</v>
       </c>
       <c r="HZ4" s="3" t="n">
         <v>8</v>
@@ -4669,10 +4669,10 @@
         <v>11.69</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>9.43</v>
+        <v>9.41</v>
       </c>
       <c r="L5" s="3" t="n">
-        <v>9.43</v>
+        <v>9.41</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>7.68</v>
@@ -4684,10 +4684,10 @@
         <v>6.24</v>
       </c>
       <c r="P5" s="3" t="n">
-        <v>9</v>
+        <v>8.99</v>
       </c>
       <c r="Q5" s="3" t="n">
-        <v>6.48</v>
+        <v>6.47</v>
       </c>
       <c r="R5" s="3" t="n">
         <v>0.72</v>
@@ -4744,19 +4744,19 @@
         <v>59.4</v>
       </c>
       <c r="AH5" s="6" t="n">
-        <v>56.5</v>
+        <v>56.4</v>
       </c>
       <c r="AI5" s="7" t="n">
-        <v>56</v>
+        <v>55.9</v>
       </c>
       <c r="AJ5" s="7" t="n">
         <v>48.6</v>
       </c>
       <c r="AK5" s="7" t="n">
-        <v>44.1</v>
+        <v>44</v>
       </c>
       <c r="AL5" s="7" t="n">
-        <v>44.1</v>
+        <v>44</v>
       </c>
       <c r="AM5" s="7" t="n">
         <v>40.4</v>
@@ -4771,34 +4771,34 @@
         <v>34.6</v>
       </c>
       <c r="AQ5" s="8" t="n">
-        <v>31.7</v>
+        <v>31.6</v>
       </c>
       <c r="AR5" s="8" t="n">
-        <v>30.3</v>
+        <v>30.1</v>
       </c>
       <c r="AS5" s="8" t="n">
-        <v>30.3</v>
+        <v>30.1</v>
       </c>
       <c r="AT5" s="8" t="n">
-        <v>26.2</v>
+        <v>26.1</v>
       </c>
       <c r="AU5" s="8" t="n">
-        <v>24.9</v>
+        <v>24.8</v>
       </c>
       <c r="AV5" s="8" t="n">
-        <v>24.9</v>
+        <v>24.8</v>
       </c>
       <c r="AW5" s="8" t="n">
-        <v>21.4</v>
+        <v>21.2</v>
       </c>
       <c r="AX5" s="8" t="n">
-        <v>19.3</v>
+        <v>19.2</v>
       </c>
       <c r="AY5" s="8" t="n">
-        <v>19.3</v>
+        <v>19.2</v>
       </c>
       <c r="AZ5" s="3" t="n">
-        <v>237.83</v>
+        <v>237.53</v>
       </c>
       <c r="BA5" s="4" t="inlineStr">
         <is>
@@ -4822,7 +4822,7 @@
         <v>59.4</v>
       </c>
       <c r="BF5" s="3" t="n">
-        <v>2.93</v>
+        <v>2.91</v>
       </c>
       <c r="BG5" s="3" t="n">
         <v>18.8</v>
@@ -5284,7 +5284,7 @@
         </is>
       </c>
       <c r="GR5" s="3" t="n">
-        <v>6.48</v>
+        <v>6.47</v>
       </c>
       <c r="GS5" s="3" t="n">
         <v>4.08</v>
@@ -5334,19 +5334,19 @@
         <v>55.9</v>
       </c>
       <c r="HH5" s="3" t="n">
-        <v>53.5</v>
+        <v>53.4</v>
       </c>
       <c r="HI5" s="3" t="n">
-        <v>53.5</v>
+        <v>53.4</v>
       </c>
       <c r="HJ5" s="3" t="n">
         <v>47.6</v>
       </c>
       <c r="HK5" s="3" t="n">
-        <v>44.1</v>
+        <v>44</v>
       </c>
       <c r="HL5" s="3" t="n">
-        <v>44.1</v>
+        <v>44</v>
       </c>
       <c r="HM5" s="3" t="n">
         <v>40.4</v>
@@ -5361,31 +5361,31 @@
         <v>34.6</v>
       </c>
       <c r="HQ5" s="3" t="n">
-        <v>31.7</v>
+        <v>31.6</v>
       </c>
       <c r="HR5" s="3" t="n">
-        <v>30.3</v>
+        <v>30.1</v>
       </c>
       <c r="HS5" s="3" t="n">
-        <v>30.3</v>
+        <v>30.1</v>
       </c>
       <c r="HT5" s="3" t="n">
-        <v>26.2</v>
+        <v>26.1</v>
       </c>
       <c r="HU5" s="3" t="n">
-        <v>24.9</v>
+        <v>24.8</v>
       </c>
       <c r="HV5" s="3" t="n">
-        <v>24.9</v>
+        <v>24.8</v>
       </c>
       <c r="HW5" s="3" t="n">
-        <v>21.4</v>
+        <v>21.2</v>
       </c>
       <c r="HX5" s="3" t="n">
-        <v>19.3</v>
+        <v>19.2</v>
       </c>
       <c r="HY5" s="3" t="n">
-        <v>19.3</v>
+        <v>19.2</v>
       </c>
       <c r="HZ5" s="3" t="n">
         <v>0</v>
@@ -5520,10 +5520,10 @@
         <v>10.66</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>9.6</v>
+        <v>9.59</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>9.6</v>
+        <v>9.59</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>8.4</v>
@@ -5601,34 +5601,34 @@
         <v>60.6</v>
       </c>
       <c r="AJ6" s="6" t="n">
-        <v>51.4</v>
+        <v>51.2</v>
       </c>
       <c r="AK6" s="7" t="n">
-        <v>45.4</v>
+        <v>45.3</v>
       </c>
       <c r="AL6" s="7" t="n">
-        <v>45.4</v>
+        <v>45.3</v>
       </c>
       <c r="AM6" s="7" t="n">
-        <v>40.8</v>
+        <v>40.6</v>
       </c>
       <c r="AN6" s="8" t="n">
-        <v>35.9</v>
+        <v>35.8</v>
       </c>
       <c r="AO6" s="8" t="n">
-        <v>35.9</v>
+        <v>35.8</v>
       </c>
       <c r="AP6" s="8" t="n">
-        <v>33.4</v>
+        <v>33.2</v>
       </c>
       <c r="AQ6" s="8" t="n">
-        <v>29.6</v>
+        <v>29.5</v>
       </c>
       <c r="AR6" s="8" t="n">
-        <v>29.6</v>
+        <v>29.5</v>
       </c>
       <c r="AS6" s="8" t="n">
-        <v>27.6</v>
+        <v>27.5</v>
       </c>
       <c r="AT6" s="8" t="n">
         <v>23</v>
@@ -5637,7 +5637,7 @@
         <v>23</v>
       </c>
       <c r="AV6" s="8" t="n">
-        <v>21.5</v>
+        <v>21.4</v>
       </c>
       <c r="AW6" s="8" t="n">
         <v>18.4</v>
@@ -5646,10 +5646,10 @@
         <v>18.4</v>
       </c>
       <c r="AY6" s="8" t="n">
-        <v>16.3</v>
+        <v>16.2</v>
       </c>
       <c r="AZ6" s="3" t="n">
-        <v>236.22</v>
+        <v>236.07</v>
       </c>
       <c r="BA6" s="4" t="inlineStr">
         <is>
@@ -5673,7 +5673,7 @@
         <v>60.6</v>
       </c>
       <c r="BF6" s="3" t="n">
-        <v>2.1</v>
+        <v>2.09</v>
       </c>
       <c r="BG6" s="3" t="n">
         <v>21.2</v>
@@ -6138,7 +6138,7 @@
         <v>5.91</v>
       </c>
       <c r="GS6" s="3" t="n">
-        <v>5.4</v>
+        <v>5.39</v>
       </c>
       <c r="GT6" s="3" t="n">
         <v>12.9</v>
@@ -6147,7 +6147,7 @@
         <v>18.16</v>
       </c>
       <c r="GV6" s="3" t="n">
-        <v>4.65</v>
+        <v>4.64</v>
       </c>
       <c r="GW6" s="3" t="n">
         <v>0</v>
@@ -6191,34 +6191,34 @@
         <v>58.1</v>
       </c>
       <c r="HJ6" s="3" t="n">
-        <v>50.4</v>
+        <v>50.2</v>
       </c>
       <c r="HK6" s="3" t="n">
-        <v>45.4</v>
+        <v>45.3</v>
       </c>
       <c r="HL6" s="3" t="n">
-        <v>45.4</v>
+        <v>45.3</v>
       </c>
       <c r="HM6" s="3" t="n">
-        <v>40.8</v>
+        <v>40.6</v>
       </c>
       <c r="HN6" s="3" t="n">
-        <v>35.9</v>
+        <v>35.8</v>
       </c>
       <c r="HO6" s="3" t="n">
-        <v>35.9</v>
+        <v>35.8</v>
       </c>
       <c r="HP6" s="3" t="n">
-        <v>33.4</v>
+        <v>33.2</v>
       </c>
       <c r="HQ6" s="3" t="n">
-        <v>29.6</v>
+        <v>29.5</v>
       </c>
       <c r="HR6" s="3" t="n">
-        <v>29.6</v>
+        <v>29.5</v>
       </c>
       <c r="HS6" s="3" t="n">
-        <v>27.6</v>
+        <v>27.5</v>
       </c>
       <c r="HT6" s="3" t="n">
         <v>23</v>
@@ -6227,7 +6227,7 @@
         <v>23</v>
       </c>
       <c r="HV6" s="3" t="n">
-        <v>21.5</v>
+        <v>21.4</v>
       </c>
       <c r="HW6" s="3" t="n">
         <v>18.4</v>
@@ -6236,7 +6236,7 @@
         <v>18.4</v>
       </c>
       <c r="HY6" s="3" t="n">
-        <v>16.3</v>
+        <v>16.2</v>
       </c>
       <c r="HZ6" s="3" t="n">
         <v>4.3</v>
@@ -6422,13 +6422,13 @@
         <v>99.5</v>
       </c>
       <c r="Z7" s="5" t="n">
-        <v>91.90000000000001</v>
+        <v>92</v>
       </c>
       <c r="AA7" s="5" t="n">
         <v>91.59999999999999</v>
       </c>
       <c r="AB7" s="5" t="n">
-        <v>91.2</v>
+        <v>91.3</v>
       </c>
       <c r="AC7" s="5" t="n">
         <v>83.2</v>
@@ -6446,13 +6446,13 @@
         <v>59.6</v>
       </c>
       <c r="AH7" s="6" t="n">
-        <v>55.2</v>
+        <v>55.3</v>
       </c>
       <c r="AI7" s="7" t="n">
-        <v>54.7</v>
+        <v>54.8</v>
       </c>
       <c r="AJ7" s="7" t="n">
-        <v>45.7</v>
+        <v>45.8</v>
       </c>
       <c r="AK7" s="7" t="n">
         <v>41.4</v>
@@ -6467,10 +6467,10 @@
         <v>33.7</v>
       </c>
       <c r="AO7" s="8" t="n">
-        <v>31.4</v>
+        <v>31.3</v>
       </c>
       <c r="AP7" s="8" t="n">
-        <v>31.4</v>
+        <v>31.3</v>
       </c>
       <c r="AQ7" s="8" t="n">
         <v>28.9</v>
@@ -6491,7 +6491,7 @@
         <v>22.4</v>
       </c>
       <c r="AW7" s="8" t="n">
-        <v>19</v>
+        <v>19.1</v>
       </c>
       <c r="AX7" s="8" t="n">
         <v>17.1</v>
@@ -6500,7 +6500,7 @@
         <v>17.1</v>
       </c>
       <c r="AZ7" s="3" t="n">
-        <v>226.72</v>
+        <v>226.73</v>
       </c>
       <c r="BA7" s="4" t="inlineStr">
         <is>
@@ -7012,13 +7012,13 @@
         <v>100</v>
       </c>
       <c r="GZ7" s="3" t="n">
-        <v>86.5</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="HA7" s="3" t="n">
-        <v>86.5</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="HB7" s="3" t="n">
-        <v>86.5</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="HC7" s="3" t="n">
         <v>77.2</v>
@@ -7036,13 +7036,13 @@
         <v>56.1</v>
       </c>
       <c r="HH7" s="3" t="n">
-        <v>52.2</v>
+        <v>52.3</v>
       </c>
       <c r="HI7" s="3" t="n">
-        <v>52.2</v>
+        <v>52.3</v>
       </c>
       <c r="HJ7" s="3" t="n">
-        <v>44.7</v>
+        <v>44.8</v>
       </c>
       <c r="HK7" s="3" t="n">
         <v>41.4</v>
@@ -7057,10 +7057,10 @@
         <v>33.7</v>
       </c>
       <c r="HO7" s="3" t="n">
-        <v>31.4</v>
+        <v>31.3</v>
       </c>
       <c r="HP7" s="3" t="n">
-        <v>31.4</v>
+        <v>31.3</v>
       </c>
       <c r="HQ7" s="3" t="n">
         <v>28.9</v>
@@ -7081,7 +7081,7 @@
         <v>22.4</v>
       </c>
       <c r="HW7" s="3" t="n">
-        <v>19</v>
+        <v>19.1</v>
       </c>
       <c r="HX7" s="3" t="n">
         <v>17.1</v>
@@ -7096,7 +7096,7 @@
         <v>5.4</v>
       </c>
       <c r="IB7" s="3" t="n">
-        <v>5.1</v>
+        <v>5</v>
       </c>
       <c r="IC7" s="3" t="n">
         <v>4.7</v>
@@ -7222,10 +7222,10 @@
         <v>9.85</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>8.949999999999999</v>
+        <v>8.960000000000001</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>8.949999999999999</v>
+        <v>8.960000000000001</v>
       </c>
       <c r="M8" s="3" t="n">
         <v>7.42</v>
@@ -7237,13 +7237,13 @@
         <v>5.87</v>
       </c>
       <c r="P8" s="3" t="n">
-        <v>7.49</v>
+        <v>7.48</v>
       </c>
       <c r="Q8" s="3" t="n">
         <v>5.87</v>
       </c>
       <c r="R8" s="3" t="n">
-        <v>0.784</v>
+        <v>0.785</v>
       </c>
       <c r="S8" s="3" t="n">
         <v>8.6</v>
@@ -7276,7 +7276,7 @@
         <v>92.8</v>
       </c>
       <c r="AA8" s="5" t="n">
-        <v>92.5</v>
+        <v>88.5</v>
       </c>
       <c r="AB8" s="5" t="n">
         <v>88</v>
@@ -7300,25 +7300,25 @@
         <v>58.4</v>
       </c>
       <c r="AI8" s="6" t="n">
-        <v>49.7</v>
+        <v>49.8</v>
       </c>
       <c r="AJ8" s="7" t="n">
-        <v>48.2</v>
+        <v>48.3</v>
       </c>
       <c r="AK8" s="7" t="n">
-        <v>41.9</v>
+        <v>42</v>
       </c>
       <c r="AL8" s="8" t="n">
-        <v>37.1</v>
+        <v>37.2</v>
       </c>
       <c r="AM8" s="8" t="n">
-        <v>37.1</v>
+        <v>37.2</v>
       </c>
       <c r="AN8" s="8" t="n">
-        <v>32.2</v>
+        <v>32.3</v>
       </c>
       <c r="AO8" s="8" t="n">
-        <v>32.2</v>
+        <v>32.3</v>
       </c>
       <c r="AP8" s="8" t="n">
         <v>29.5</v>
@@ -7330,13 +7330,13 @@
         <v>25.9</v>
       </c>
       <c r="AS8" s="8" t="n">
-        <v>23.8</v>
+        <v>23.9</v>
       </c>
       <c r="AT8" s="8" t="n">
-        <v>20.3</v>
+        <v>20.4</v>
       </c>
       <c r="AU8" s="8" t="n">
-        <v>20.3</v>
+        <v>20.4</v>
       </c>
       <c r="AV8" s="8" t="n">
         <v>18.9</v>
@@ -7351,7 +7351,7 @@
         <v>13.9</v>
       </c>
       <c r="AZ8" s="3" t="n">
-        <v>226.31</v>
+        <v>226.47</v>
       </c>
       <c r="BA8" s="4" t="inlineStr">
         <is>
@@ -7360,7 +7360,7 @@
       </c>
       <c r="BB8" s="9" t="inlineStr">
         <is>
-          <t>MORE 7.0 | 58.4% | Edge +1.9</t>
+          <t>MORE 7.0 | 58.4% | Edge +2.0</t>
         </is>
       </c>
       <c r="BC8" s="4" t="inlineStr">
@@ -7375,7 +7375,7 @@
         <v>58.4</v>
       </c>
       <c r="BF8" s="3" t="n">
-        <v>1.95</v>
+        <v>1.96</v>
       </c>
       <c r="BG8" s="3" t="n">
         <v>16.8</v>
@@ -7840,13 +7840,13 @@
         <v>5.87</v>
       </c>
       <c r="GS8" s="3" t="n">
-        <v>4.29</v>
+        <v>4.28</v>
       </c>
       <c r="GT8" s="3" t="n">
-        <v>12.12</v>
+        <v>12.13</v>
       </c>
       <c r="GU8" s="3" t="n">
-        <v>17.61</v>
+        <v>17.62</v>
       </c>
       <c r="GV8" s="3" t="n">
         <v>4.58</v>
@@ -7866,7 +7866,7 @@
         <v>88</v>
       </c>
       <c r="HA8" s="3" t="n">
-        <v>88</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="HB8" s="3" t="n">
         <v>81.59999999999999</v>
@@ -7890,25 +7890,25 @@
         <v>55.4</v>
       </c>
       <c r="HI8" s="3" t="n">
-        <v>47.2</v>
+        <v>47.3</v>
       </c>
       <c r="HJ8" s="3" t="n">
-        <v>47.2</v>
+        <v>47.3</v>
       </c>
       <c r="HK8" s="3" t="n">
-        <v>41.9</v>
+        <v>42</v>
       </c>
       <c r="HL8" s="3" t="n">
-        <v>37.1</v>
+        <v>37.2</v>
       </c>
       <c r="HM8" s="3" t="n">
-        <v>37.1</v>
+        <v>37.2</v>
       </c>
       <c r="HN8" s="3" t="n">
-        <v>32.2</v>
+        <v>32.3</v>
       </c>
       <c r="HO8" s="3" t="n">
-        <v>32.2</v>
+        <v>32.3</v>
       </c>
       <c r="HP8" s="3" t="n">
         <v>29.5</v>
@@ -7920,13 +7920,13 @@
         <v>25.9</v>
       </c>
       <c r="HS8" s="3" t="n">
-        <v>23.8</v>
+        <v>23.9</v>
       </c>
       <c r="HT8" s="3" t="n">
-        <v>20.3</v>
+        <v>20.4</v>
       </c>
       <c r="HU8" s="3" t="n">
-        <v>20.3</v>
+        <v>20.4</v>
       </c>
       <c r="HV8" s="3" t="n">
         <v>18.9</v>
@@ -7947,7 +7947,7 @@
         <v>4.8</v>
       </c>
       <c r="IB8" s="3" t="n">
-        <v>4.5</v>
+        <v>6.9</v>
       </c>
       <c r="IC8" s="3" t="n">
         <v>6.4</v>
@@ -8121,10 +8121,10 @@
         </is>
       </c>
       <c r="Y9" s="5" t="n">
-        <v>91.5</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="Z9" s="5" t="n">
-        <v>91.5</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="AA9" s="5" t="n">
         <v>91.09999999999999</v>
@@ -8711,13 +8711,13 @@
         </is>
       </c>
       <c r="GY9" s="3" t="n">
-        <v>85.8</v>
+        <v>85.7</v>
       </c>
       <c r="GZ9" s="3" t="n">
-        <v>85.8</v>
+        <v>85.7</v>
       </c>
       <c r="HA9" s="3" t="n">
-        <v>85.8</v>
+        <v>85.7</v>
       </c>
       <c r="HB9" s="3" t="n">
         <v>74.7</v>
@@ -8798,7 +8798,7 @@
         <v>5.7</v>
       </c>
       <c r="IB9" s="3" t="n">
-        <v>5.3</v>
+        <v>5.4</v>
       </c>
       <c r="IC9" s="3" t="n">
         <v>7</v>
@@ -10610,13 +10610,13 @@
         <v>10.13</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>7.77</v>
+        <v>7.79</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>7.77</v>
+        <v>7.79</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>5.76</v>
+        <v>5.77</v>
       </c>
       <c r="N12" s="3" t="n">
         <v>5.6</v>
@@ -10658,46 +10658,46 @@
         </is>
       </c>
       <c r="Y12" s="5" t="n">
-        <v>84</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="Z12" s="5" t="n">
-        <v>84</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="AA12" s="5" t="n">
-        <v>83.5</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="AB12" s="5" t="n">
-        <v>75.8</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="AC12" s="5" t="n">
-        <v>67</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="AD12" s="5" t="n">
-        <v>66</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="AE12" s="5" t="n">
         <v>61.7</v>
       </c>
       <c r="AF12" s="6" t="n">
-        <v>52.7</v>
+        <v>52.8</v>
       </c>
       <c r="AG12" s="7" t="n">
-        <v>49.7</v>
+        <v>49.8</v>
       </c>
       <c r="AH12" s="7" t="n">
-        <v>49.2</v>
+        <v>49.3</v>
       </c>
       <c r="AI12" s="7" t="n">
-        <v>41.3</v>
+        <v>41.4</v>
       </c>
       <c r="AJ12" s="8" t="n">
-        <v>36.3</v>
+        <v>36.4</v>
       </c>
       <c r="AK12" s="8" t="n">
-        <v>35.3</v>
+        <v>35.4</v>
       </c>
       <c r="AL12" s="8" t="n">
-        <v>31.6</v>
+        <v>31.7</v>
       </c>
       <c r="AM12" s="8" t="n">
         <v>28.1</v>
@@ -10709,37 +10709,37 @@
         <v>26.2</v>
       </c>
       <c r="AP12" s="8" t="n">
-        <v>23.8</v>
+        <v>23.9</v>
       </c>
       <c r="AQ12" s="8" t="n">
-        <v>23.8</v>
+        <v>23.9</v>
       </c>
       <c r="AR12" s="8" t="n">
-        <v>22.7</v>
+        <v>22.8</v>
       </c>
       <c r="AS12" s="8" t="n">
-        <v>18.9</v>
+        <v>19</v>
       </c>
       <c r="AT12" s="8" t="n">
-        <v>18.9</v>
+        <v>19</v>
       </c>
       <c r="AU12" s="8" t="n">
-        <v>18.1</v>
+        <v>18.2</v>
       </c>
       <c r="AV12" s="8" t="n">
-        <v>14.9</v>
+        <v>15</v>
       </c>
       <c r="AW12" s="8" t="n">
-        <v>13.2</v>
+        <v>13.4</v>
       </c>
       <c r="AX12" s="8" t="n">
-        <v>13.2</v>
+        <v>13.4</v>
       </c>
       <c r="AY12" s="8" t="n">
-        <v>11.4</v>
+        <v>11.5</v>
       </c>
       <c r="AZ12" s="3" t="n">
-        <v>206.35</v>
+        <v>206.67</v>
       </c>
       <c r="BA12" s="4" t="inlineStr">
         <is>
@@ -10763,7 +10763,7 @@
         <v>61.7</v>
       </c>
       <c r="BF12" s="3" t="n">
-        <v>2.27</v>
+        <v>2.29</v>
       </c>
       <c r="BG12" s="3" t="n">
         <v>23.4</v>
@@ -11234,7 +11234,7 @@
         <v>10.84</v>
       </c>
       <c r="GU12" s="3" t="n">
-        <v>15.91</v>
+        <v>15.92</v>
       </c>
       <c r="GV12" s="3" t="n">
         <v>3.86</v>
@@ -11248,46 +11248,46 @@
         </is>
       </c>
       <c r="GY12" s="3" t="n">
-        <v>76</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="GZ12" s="3" t="n">
-        <v>76</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="HA12" s="3" t="n">
-        <v>76</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="HB12" s="3" t="n">
-        <v>68.8</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="HC12" s="3" t="n">
-        <v>61</v>
+        <v>61.1</v>
       </c>
       <c r="HD12" s="3" t="n">
-        <v>61</v>
+        <v>61.1</v>
       </c>
       <c r="HE12" s="3" t="n">
         <v>57.2</v>
       </c>
       <c r="HF12" s="3" t="n">
-        <v>48.7</v>
+        <v>48.8</v>
       </c>
       <c r="HG12" s="3" t="n">
-        <v>46.2</v>
+        <v>46.3</v>
       </c>
       <c r="HH12" s="3" t="n">
-        <v>46.2</v>
+        <v>46.3</v>
       </c>
       <c r="HI12" s="3" t="n">
-        <v>38.8</v>
+        <v>38.9</v>
       </c>
       <c r="HJ12" s="3" t="n">
-        <v>35.3</v>
+        <v>35.4</v>
       </c>
       <c r="HK12" s="3" t="n">
-        <v>35.3</v>
+        <v>35.4</v>
       </c>
       <c r="HL12" s="3" t="n">
-        <v>31.6</v>
+        <v>31.7</v>
       </c>
       <c r="HM12" s="3" t="n">
         <v>28.1</v>
@@ -11299,34 +11299,34 @@
         <v>26.2</v>
       </c>
       <c r="HP12" s="3" t="n">
-        <v>23.8</v>
+        <v>23.9</v>
       </c>
       <c r="HQ12" s="3" t="n">
-        <v>23.8</v>
+        <v>23.9</v>
       </c>
       <c r="HR12" s="3" t="n">
-        <v>22.7</v>
+        <v>22.8</v>
       </c>
       <c r="HS12" s="3" t="n">
-        <v>18.9</v>
+        <v>19</v>
       </c>
       <c r="HT12" s="3" t="n">
-        <v>18.9</v>
+        <v>19</v>
       </c>
       <c r="HU12" s="3" t="n">
-        <v>18.1</v>
+        <v>18.2</v>
       </c>
       <c r="HV12" s="3" t="n">
-        <v>14.9</v>
+        <v>15</v>
       </c>
       <c r="HW12" s="3" t="n">
-        <v>13.2</v>
+        <v>13.4</v>
       </c>
       <c r="HX12" s="3" t="n">
-        <v>13.2</v>
+        <v>13.4</v>
       </c>
       <c r="HY12" s="3" t="n">
-        <v>11.4</v>
+        <v>11.5</v>
       </c>
       <c r="HZ12" s="3" t="n">
         <v>8</v>
@@ -11461,10 +11461,10 @@
         <v>9.74</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>7.77</v>
+        <v>7.76</v>
       </c>
       <c r="L13" s="3" t="n">
-        <v>7.77</v>
+        <v>7.76</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>6.26</v>
@@ -11509,7 +11509,7 @@
         </is>
       </c>
       <c r="Y13" s="5" t="n">
-        <v>84.59999999999999</v>
+        <v>84.5</v>
       </c>
       <c r="Z13" s="5" t="n">
         <v>78.8</v>
@@ -11524,7 +11524,7 @@
         <v>69.5</v>
       </c>
       <c r="AD13" s="5" t="n">
-        <v>64.2</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="AE13" s="6" t="n">
         <v>55</v>
@@ -11560,13 +11560,13 @@
         <v>28.3</v>
       </c>
       <c r="AP13" s="8" t="n">
-        <v>25.5</v>
+        <v>25.6</v>
       </c>
       <c r="AQ13" s="8" t="n">
-        <v>22.7</v>
+        <v>22.8</v>
       </c>
       <c r="AR13" s="8" t="n">
-        <v>22.7</v>
+        <v>22.8</v>
       </c>
       <c r="AS13" s="8" t="n">
         <v>21</v>
@@ -11575,7 +11575,7 @@
         <v>21</v>
       </c>
       <c r="AU13" s="8" t="n">
-        <v>17.3</v>
+        <v>17.2</v>
       </c>
       <c r="AV13" s="8" t="n">
         <v>16</v>
@@ -11590,7 +11590,7 @@
         <v>13.8</v>
       </c>
       <c r="AZ13" s="3" t="n">
-        <v>206.22</v>
+        <v>206.08</v>
       </c>
       <c r="BA13" s="4" t="inlineStr">
         <is>
@@ -11599,7 +11599,7 @@
       </c>
       <c r="BB13" s="9" t="inlineStr">
         <is>
-          <t>MORE 5.0 | 64.2% | Edge +2.8</t>
+          <t>MORE 5.0 | 64.1% | Edge +2.8</t>
         </is>
       </c>
       <c r="BC13" s="4" t="inlineStr">
@@ -11611,13 +11611,13 @@
         <v>5</v>
       </c>
       <c r="BE13" s="3" t="n">
-        <v>64.2</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="BF13" s="3" t="n">
-        <v>2.77</v>
+        <v>2.76</v>
       </c>
       <c r="BG13" s="3" t="n">
-        <v>28.4</v>
+        <v>28.2</v>
       </c>
       <c r="BH13" s="4" t="inlineStr">
         <is>
@@ -12085,7 +12085,7 @@
         <v>11.37</v>
       </c>
       <c r="GU13" s="3" t="n">
-        <v>17.33</v>
+        <v>17.34</v>
       </c>
       <c r="GV13" s="3" t="n">
         <v>4.07</v>
@@ -12099,7 +12099,7 @@
         </is>
       </c>
       <c r="GY13" s="3" t="n">
-        <v>76.59999999999999</v>
+        <v>76.5</v>
       </c>
       <c r="GZ13" s="3" t="n">
         <v>70.8</v>
@@ -12114,7 +12114,7 @@
         <v>63.5</v>
       </c>
       <c r="HD13" s="3" t="n">
-        <v>59.2</v>
+        <v>59.1</v>
       </c>
       <c r="HE13" s="3" t="n">
         <v>50.5</v>
@@ -12150,13 +12150,13 @@
         <v>28.3</v>
       </c>
       <c r="HP13" s="3" t="n">
-        <v>25.5</v>
+        <v>25.6</v>
       </c>
       <c r="HQ13" s="3" t="n">
-        <v>22.7</v>
+        <v>22.8</v>
       </c>
       <c r="HR13" s="3" t="n">
-        <v>22.7</v>
+        <v>22.8</v>
       </c>
       <c r="HS13" s="3" t="n">
         <v>21</v>
@@ -12165,7 +12165,7 @@
         <v>21</v>
       </c>
       <c r="HU13" s="3" t="n">
-        <v>17.3</v>
+        <v>17.2</v>
       </c>
       <c r="HV13" s="3" t="n">
         <v>16</v>
@@ -12312,10 +12312,10 @@
         <v>8.92</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>8.449999999999999</v>
+        <v>8.460000000000001</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>8.449999999999999</v>
+        <v>8.460000000000001</v>
       </c>
       <c r="M14" s="3" t="n">
         <v>6</v>
@@ -12381,16 +12381,16 @@
         <v>57.4</v>
       </c>
       <c r="AF14" s="7" t="n">
-        <v>53.2</v>
+        <v>53.3</v>
       </c>
       <c r="AG14" s="7" t="n">
-        <v>52.7</v>
+        <v>52.8</v>
       </c>
       <c r="AH14" s="7" t="n">
-        <v>45.5</v>
+        <v>45.6</v>
       </c>
       <c r="AI14" s="7" t="n">
-        <v>45</v>
+        <v>45.1</v>
       </c>
       <c r="AJ14" s="8" t="n">
         <v>39</v>
@@ -12399,49 +12399,49 @@
         <v>38</v>
       </c>
       <c r="AL14" s="8" t="n">
-        <v>34.1</v>
+        <v>34.2</v>
       </c>
       <c r="AM14" s="8" t="n">
-        <v>34.1</v>
+        <v>34.2</v>
       </c>
       <c r="AN14" s="8" t="n">
-        <v>30.4</v>
+        <v>30.5</v>
       </c>
       <c r="AO14" s="8" t="n">
-        <v>30.4</v>
+        <v>30.5</v>
       </c>
       <c r="AP14" s="8" t="n">
-        <v>28.6</v>
+        <v>28.7</v>
       </c>
       <c r="AQ14" s="8" t="n">
-        <v>28.6</v>
+        <v>28.7</v>
       </c>
       <c r="AR14" s="8" t="n">
-        <v>25.8</v>
+        <v>25.9</v>
       </c>
       <c r="AS14" s="8" t="n">
-        <v>25.8</v>
+        <v>25.9</v>
       </c>
       <c r="AT14" s="8" t="n">
-        <v>24.4</v>
+        <v>24.6</v>
       </c>
       <c r="AU14" s="8" t="n">
-        <v>24.4</v>
+        <v>24.6</v>
       </c>
       <c r="AV14" s="8" t="n">
-        <v>19.8</v>
+        <v>19.9</v>
       </c>
       <c r="AW14" s="8" t="n">
-        <v>19.8</v>
+        <v>19.9</v>
       </c>
       <c r="AX14" s="8" t="n">
-        <v>18.7</v>
+        <v>18.8</v>
       </c>
       <c r="AY14" s="8" t="n">
-        <v>18.7</v>
+        <v>18.8</v>
       </c>
       <c r="AZ14" s="3" t="n">
-        <v>205.51</v>
+        <v>205.67</v>
       </c>
       <c r="BA14" s="4" t="inlineStr">
         <is>
@@ -12450,7 +12450,7 @@
       </c>
       <c r="BB14" s="9" t="inlineStr">
         <is>
-          <t>MORE 4.5 | 69.0% | Edge +3.9</t>
+          <t>MORE 4.5 | 69.0% | Edge +4.0</t>
         </is>
       </c>
       <c r="BC14" s="4" t="inlineStr">
@@ -12465,7 +12465,7 @@
         <v>69</v>
       </c>
       <c r="BF14" s="3" t="n">
-        <v>3.95</v>
+        <v>3.96</v>
       </c>
       <c r="BG14" s="3" t="n">
         <v>38</v>
@@ -12971,16 +12971,16 @@
         <v>57.4</v>
       </c>
       <c r="HF14" s="3" t="n">
-        <v>53.2</v>
+        <v>53.3</v>
       </c>
       <c r="HG14" s="3" t="n">
-        <v>52.7</v>
+        <v>52.8</v>
       </c>
       <c r="HH14" s="3" t="n">
-        <v>45.5</v>
+        <v>45.6</v>
       </c>
       <c r="HI14" s="3" t="n">
-        <v>45</v>
+        <v>45.1</v>
       </c>
       <c r="HJ14" s="3" t="n">
         <v>39</v>
@@ -12989,46 +12989,46 @@
         <v>38</v>
       </c>
       <c r="HL14" s="3" t="n">
-        <v>34.1</v>
+        <v>34.2</v>
       </c>
       <c r="HM14" s="3" t="n">
-        <v>34.1</v>
+        <v>34.2</v>
       </c>
       <c r="HN14" s="3" t="n">
-        <v>30.4</v>
+        <v>30.5</v>
       </c>
       <c r="HO14" s="3" t="n">
-        <v>30.4</v>
+        <v>30.5</v>
       </c>
       <c r="HP14" s="3" t="n">
-        <v>28.6</v>
+        <v>28.7</v>
       </c>
       <c r="HQ14" s="3" t="n">
-        <v>28.6</v>
+        <v>28.7</v>
       </c>
       <c r="HR14" s="3" t="n">
-        <v>25.8</v>
+        <v>25.9</v>
       </c>
       <c r="HS14" s="3" t="n">
-        <v>25.8</v>
+        <v>25.9</v>
       </c>
       <c r="HT14" s="3" t="n">
-        <v>24.4</v>
+        <v>24.6</v>
       </c>
       <c r="HU14" s="3" t="n">
-        <v>24.4</v>
+        <v>24.6</v>
       </c>
       <c r="HV14" s="3" t="n">
-        <v>19.8</v>
+        <v>19.9</v>
       </c>
       <c r="HW14" s="3" t="n">
-        <v>19.8</v>
+        <v>19.9</v>
       </c>
       <c r="HX14" s="3" t="n">
-        <v>18.7</v>
+        <v>18.8</v>
       </c>
       <c r="HY14" s="3" t="n">
-        <v>18.7</v>
+        <v>18.8</v>
       </c>
       <c r="HZ14" s="4" t="n"/>
       <c r="IA14" s="4" t="n"/>
@@ -13109,10 +13109,10 @@
         <v>9.470000000000001</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>7.38</v>
+        <v>7.37</v>
       </c>
       <c r="L15" s="3" t="n">
-        <v>7.38</v>
+        <v>7.37</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>4.33</v>
@@ -13124,13 +13124,13 @@
         <v>7.87</v>
       </c>
       <c r="P15" s="3" t="n">
-        <v>6.66</v>
+        <v>6.65</v>
       </c>
       <c r="Q15" s="3" t="n">
         <v>7.63</v>
       </c>
       <c r="R15" s="3" t="n">
-        <v>1.182</v>
+        <v>1.183</v>
       </c>
       <c r="S15" s="3" t="n">
         <v>4.6</v>
@@ -13190,13 +13190,13 @@
         <v>40</v>
       </c>
       <c r="AJ15" s="8" t="n">
-        <v>33.8</v>
+        <v>33.7</v>
       </c>
       <c r="AK15" s="8" t="n">
-        <v>32.8</v>
+        <v>32.7</v>
       </c>
       <c r="AL15" s="8" t="n">
-        <v>32.8</v>
+        <v>32.7</v>
       </c>
       <c r="AM15" s="8" t="n">
         <v>28.7</v>
@@ -13211,13 +13211,13 @@
         <v>24.2</v>
       </c>
       <c r="AQ15" s="8" t="n">
-        <v>21.9</v>
+        <v>21.8</v>
       </c>
       <c r="AR15" s="8" t="n">
-        <v>21.9</v>
+        <v>21.8</v>
       </c>
       <c r="AS15" s="8" t="n">
-        <v>21.9</v>
+        <v>21.8</v>
       </c>
       <c r="AT15" s="8" t="n">
         <v>19.1</v>
@@ -13232,13 +13232,13 @@
         <v>17.3</v>
       </c>
       <c r="AX15" s="8" t="n">
-        <v>14.1</v>
+        <v>14</v>
       </c>
       <c r="AY15" s="8" t="n">
-        <v>14.1</v>
+        <v>14</v>
       </c>
       <c r="AZ15" s="3" t="n">
-        <v>205</v>
+        <v>204.85</v>
       </c>
       <c r="BA15" s="4" t="inlineStr">
         <is>
@@ -13262,7 +13262,7 @@
         <v>68.09999999999999</v>
       </c>
       <c r="BF15" s="3" t="n">
-        <v>3.38</v>
+        <v>3.37</v>
       </c>
       <c r="BG15" s="3" t="n">
         <v>36.2</v>
@@ -13733,7 +13733,7 @@
         <v>10.25</v>
       </c>
       <c r="GU15" s="3" t="n">
-        <v>18.52</v>
+        <v>18.53</v>
       </c>
       <c r="GV15" s="3" t="n">
         <v>4.32</v>
@@ -13780,13 +13780,13 @@
         <v>37.5</v>
       </c>
       <c r="HJ15" s="3" t="n">
-        <v>32.8</v>
+        <v>32.7</v>
       </c>
       <c r="HK15" s="3" t="n">
-        <v>32.8</v>
+        <v>32.7</v>
       </c>
       <c r="HL15" s="3" t="n">
-        <v>32.8</v>
+        <v>32.7</v>
       </c>
       <c r="HM15" s="3" t="n">
         <v>28.7</v>
@@ -13801,13 +13801,13 @@
         <v>24.2</v>
       </c>
       <c r="HQ15" s="3" t="n">
-        <v>21.9</v>
+        <v>21.8</v>
       </c>
       <c r="HR15" s="3" t="n">
-        <v>21.9</v>
+        <v>21.8</v>
       </c>
       <c r="HS15" s="3" t="n">
-        <v>21.9</v>
+        <v>21.8</v>
       </c>
       <c r="HT15" s="3" t="n">
         <v>19.1</v>
@@ -13822,10 +13822,10 @@
         <v>17.3</v>
       </c>
       <c r="HX15" s="3" t="n">
-        <v>14.1</v>
+        <v>14</v>
       </c>
       <c r="HY15" s="3" t="n">
-        <v>14.1</v>
+        <v>14</v>
       </c>
       <c r="HZ15" s="3" t="n">
         <v>8</v>
@@ -13960,10 +13960,10 @@
         <v>8.529999999999999</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>7.83</v>
+        <v>7.82</v>
       </c>
       <c r="L16" s="3" t="n">
-        <v>7.83</v>
+        <v>7.82</v>
       </c>
       <c r="M16" s="3" t="n">
         <v>5</v>
@@ -13975,10 +13975,10 @@
         <v>7.14</v>
       </c>
       <c r="P16" s="3" t="n">
-        <v>7.25</v>
+        <v>7.24</v>
       </c>
       <c r="Q16" s="3" t="n">
-        <v>7.25</v>
+        <v>7.24</v>
       </c>
       <c r="R16" s="3" t="n">
         <v>1</v>
@@ -14017,16 +14017,16 @@
         <v>72.8</v>
       </c>
       <c r="AB16" s="5" t="n">
-        <v>67.90000000000001</v>
+        <v>67.8</v>
       </c>
       <c r="AC16" s="5" t="n">
-        <v>66.90000000000001</v>
+        <v>66.8</v>
       </c>
       <c r="AD16" s="6" t="n">
-        <v>54.5</v>
+        <v>54.4</v>
       </c>
       <c r="AE16" s="7" t="n">
-        <v>54</v>
+        <v>53.9</v>
       </c>
       <c r="AF16" s="7" t="n">
         <v>50.1</v>
@@ -14041,10 +14041,10 @@
         <v>41.6</v>
       </c>
       <c r="AJ16" s="8" t="n">
-        <v>35.5</v>
+        <v>35.4</v>
       </c>
       <c r="AK16" s="8" t="n">
-        <v>34.5</v>
+        <v>34.4</v>
       </c>
       <c r="AL16" s="8" t="n">
         <v>31.4</v>
@@ -14071,10 +14071,10 @@
         <v>22.7</v>
       </c>
       <c r="AT16" s="8" t="n">
-        <v>21.5</v>
+        <v>21.4</v>
       </c>
       <c r="AU16" s="8" t="n">
-        <v>21.5</v>
+        <v>21.4</v>
       </c>
       <c r="AV16" s="8" t="n">
         <v>17.1</v>
@@ -14089,7 +14089,7 @@
         <v>16.1</v>
       </c>
       <c r="AZ16" s="3" t="n">
-        <v>204.76</v>
+        <v>204.61</v>
       </c>
       <c r="BA16" s="4" t="inlineStr">
         <is>
@@ -14098,7 +14098,7 @@
       </c>
       <c r="BB16" s="9" t="inlineStr">
         <is>
-          <t>MORE 4.5 | 66.9% | Edge +3.3</t>
+          <t>MORE 4.5 | 66.8% | Edge +3.3</t>
         </is>
       </c>
       <c r="BC16" s="4" t="inlineStr">
@@ -14110,13 +14110,13 @@
         <v>4.5</v>
       </c>
       <c r="BE16" s="3" t="n">
-        <v>66.90000000000001</v>
+        <v>66.8</v>
       </c>
       <c r="BF16" s="3" t="n">
-        <v>3.33</v>
+        <v>3.32</v>
       </c>
       <c r="BG16" s="3" t="n">
-        <v>33.8</v>
+        <v>33.6</v>
       </c>
       <c r="BH16" s="4" t="inlineStr">
         <is>
@@ -14575,7 +14575,7 @@
         </is>
       </c>
       <c r="GR16" s="3" t="n">
-        <v>7.25</v>
+        <v>7.24</v>
       </c>
       <c r="GS16" s="3" t="n">
         <v>3</v>
@@ -14607,16 +14607,16 @@
         <v>72.8</v>
       </c>
       <c r="HB16" s="3" t="n">
-        <v>67.90000000000001</v>
+        <v>67.8</v>
       </c>
       <c r="HC16" s="3" t="n">
-        <v>66.90000000000001</v>
+        <v>66.8</v>
       </c>
       <c r="HD16" s="3" t="n">
-        <v>54.5</v>
+        <v>54.4</v>
       </c>
       <c r="HE16" s="3" t="n">
-        <v>54</v>
+        <v>53.9</v>
       </c>
       <c r="HF16" s="3" t="n">
         <v>50.1</v>
@@ -14631,10 +14631,10 @@
         <v>41.6</v>
       </c>
       <c r="HJ16" s="3" t="n">
-        <v>35.5</v>
+        <v>35.4</v>
       </c>
       <c r="HK16" s="3" t="n">
-        <v>34.5</v>
+        <v>34.4</v>
       </c>
       <c r="HL16" s="3" t="n">
         <v>31.4</v>
@@ -14661,10 +14661,10 @@
         <v>22.7</v>
       </c>
       <c r="HT16" s="3" t="n">
-        <v>21.5</v>
+        <v>21.4</v>
       </c>
       <c r="HU16" s="3" t="n">
-        <v>21.5</v>
+        <v>21.4</v>
       </c>
       <c r="HV16" s="3" t="n">
         <v>17.1</v>
@@ -14757,10 +14757,10 @@
         <v>11.4</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>7.71</v>
+        <v>7.72</v>
       </c>
       <c r="L17" s="3" t="n">
-        <v>7.71</v>
+        <v>7.72</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>5.76</v>
@@ -14805,34 +14805,34 @@
         </is>
       </c>
       <c r="Y17" s="5" t="n">
-        <v>77.5</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="Z17" s="5" t="n">
-        <v>77.5</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="AA17" s="5" t="n">
-        <v>77</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="AB17" s="5" t="n">
-        <v>73.3</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="AC17" s="5" t="n">
-        <v>64.59999999999999</v>
+        <v>64.8</v>
       </c>
       <c r="AD17" s="5" t="n">
-        <v>63.6</v>
+        <v>63.8</v>
       </c>
       <c r="AE17" s="5" t="n">
-        <v>61.1</v>
+        <v>61.2</v>
       </c>
       <c r="AF17" s="6" t="n">
-        <v>52.2</v>
+        <v>52.3</v>
       </c>
       <c r="AG17" s="7" t="n">
-        <v>48.7</v>
+        <v>48.8</v>
       </c>
       <c r="AH17" s="7" t="n">
-        <v>48.2</v>
+        <v>48.3</v>
       </c>
       <c r="AI17" s="7" t="n">
         <v>42.3</v>
@@ -14853,7 +14853,7 @@
         <v>28.9</v>
       </c>
       <c r="AO17" s="8" t="n">
-        <v>27.1</v>
+        <v>27</v>
       </c>
       <c r="AP17" s="8" t="n">
         <v>24.3</v>
@@ -14862,7 +14862,7 @@
         <v>24.3</v>
       </c>
       <c r="AR17" s="8" t="n">
-        <v>22.8</v>
+        <v>22.7</v>
       </c>
       <c r="AS17" s="8" t="n">
         <v>19.3</v>
@@ -14886,7 +14886,7 @@
         <v>12.3</v>
       </c>
       <c r="AZ17" s="3" t="n">
-        <v>201.55</v>
+        <v>201.7</v>
       </c>
       <c r="BA17" s="4" t="inlineStr">
         <is>
@@ -14895,7 +14895,7 @@
       </c>
       <c r="BB17" s="9" t="inlineStr">
         <is>
-          <t>MORE 5.5 | 61.1% | Edge +2.2</t>
+          <t>MORE 5.5 | 61.2% | Edge +2.2</t>
         </is>
       </c>
       <c r="BC17" s="4" t="inlineStr">
@@ -14907,13 +14907,13 @@
         <v>5.5</v>
       </c>
       <c r="BE17" s="3" t="n">
-        <v>61.1</v>
+        <v>61.2</v>
       </c>
       <c r="BF17" s="3" t="n">
-        <v>2.21</v>
+        <v>2.22</v>
       </c>
       <c r="BG17" s="3" t="n">
-        <v>22.2</v>
+        <v>22.4</v>
       </c>
       <c r="BH17" s="4" t="inlineStr">
         <is>
@@ -15387,7 +15387,7 @@
         <v>3.53</v>
       </c>
       <c r="GW17" s="3" t="n">
-        <v>21.5</v>
+        <v>21.4</v>
       </c>
       <c r="GX17" s="4" t="inlineStr">
         <is>
@@ -15395,34 +15395,34 @@
         </is>
       </c>
       <c r="GY17" s="3" t="n">
-        <v>69.5</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="GZ17" s="3" t="n">
-        <v>69.5</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="HA17" s="3" t="n">
-        <v>69.5</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="HB17" s="3" t="n">
-        <v>66.3</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="HC17" s="3" t="n">
-        <v>58.6</v>
+        <v>58.8</v>
       </c>
       <c r="HD17" s="3" t="n">
-        <v>58.6</v>
+        <v>58.8</v>
       </c>
       <c r="HE17" s="3" t="n">
-        <v>56.6</v>
+        <v>56.7</v>
       </c>
       <c r="HF17" s="3" t="n">
-        <v>48.2</v>
+        <v>48.3</v>
       </c>
       <c r="HG17" s="3" t="n">
-        <v>45.2</v>
+        <v>45.3</v>
       </c>
       <c r="HH17" s="3" t="n">
-        <v>45.2</v>
+        <v>45.3</v>
       </c>
       <c r="HI17" s="3" t="n">
         <v>39.8</v>
@@ -15443,7 +15443,7 @@
         <v>28.9</v>
       </c>
       <c r="HO17" s="3" t="n">
-        <v>27.1</v>
+        <v>27</v>
       </c>
       <c r="HP17" s="3" t="n">
         <v>24.3</v>
@@ -15452,7 +15452,7 @@
         <v>24.3</v>
       </c>
       <c r="HR17" s="3" t="n">
-        <v>22.8</v>
+        <v>22.7</v>
       </c>
       <c r="HS17" s="3" t="n">
         <v>19.3</v>
@@ -16459,10 +16459,10 @@
         <v>8.550000000000001</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>7.08</v>
+        <v>7.07</v>
       </c>
       <c r="L19" s="3" t="n">
-        <v>7.08</v>
+        <v>7.07</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>5</v>
@@ -16516,16 +16516,16 @@
         <v>69.09999999999999</v>
       </c>
       <c r="AB19" s="5" t="n">
-        <v>65</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="AC19" s="5" t="n">
-        <v>64</v>
+        <v>63.9</v>
       </c>
       <c r="AD19" s="6" t="n">
-        <v>51.1</v>
+        <v>51</v>
       </c>
       <c r="AE19" s="7" t="n">
-        <v>50.6</v>
+        <v>50.5</v>
       </c>
       <c r="AF19" s="7" t="n">
         <v>46.2</v>
@@ -16546,22 +16546,22 @@
         <v>31.2</v>
       </c>
       <c r="AL19" s="8" t="n">
-        <v>27.7</v>
+        <v>27.6</v>
       </c>
       <c r="AM19" s="8" t="n">
-        <v>27.7</v>
+        <v>27.6</v>
       </c>
       <c r="AN19" s="8" t="n">
-        <v>23.9</v>
+        <v>23.8</v>
       </c>
       <c r="AO19" s="8" t="n">
-        <v>23.9</v>
+        <v>23.8</v>
       </c>
       <c r="AP19" s="8" t="n">
-        <v>22.1</v>
+        <v>22</v>
       </c>
       <c r="AQ19" s="8" t="n">
-        <v>22.1</v>
+        <v>22</v>
       </c>
       <c r="AR19" s="8" t="n">
         <v>19.7</v>
@@ -16588,7 +16588,7 @@
         <v>13</v>
       </c>
       <c r="AZ19" s="3" t="n">
-        <v>195.64</v>
+        <v>195.5</v>
       </c>
       <c r="BA19" s="4" t="inlineStr">
         <is>
@@ -16597,7 +16597,7 @@
       </c>
       <c r="BB19" s="9" t="inlineStr">
         <is>
-          <t>MORE 4.5 | 64.0% | Edge +2.6</t>
+          <t>MORE 4.5 | 63.9% | Edge +2.6</t>
         </is>
       </c>
       <c r="BC19" s="4" t="inlineStr">
@@ -16609,13 +16609,13 @@
         <v>4.5</v>
       </c>
       <c r="BE19" s="3" t="n">
-        <v>64</v>
+        <v>63.9</v>
       </c>
       <c r="BF19" s="3" t="n">
-        <v>2.58</v>
+        <v>2.57</v>
       </c>
       <c r="BG19" s="3" t="n">
-        <v>28</v>
+        <v>27.8</v>
       </c>
       <c r="BH19" s="4" t="inlineStr">
         <is>
@@ -17106,16 +17106,16 @@
         <v>69.09999999999999</v>
       </c>
       <c r="HB19" s="3" t="n">
-        <v>65</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="HC19" s="3" t="n">
-        <v>64</v>
+        <v>63.9</v>
       </c>
       <c r="HD19" s="3" t="n">
-        <v>51.1</v>
+        <v>51</v>
       </c>
       <c r="HE19" s="3" t="n">
-        <v>50.6</v>
+        <v>50.5</v>
       </c>
       <c r="HF19" s="3" t="n">
         <v>46.2</v>
@@ -17136,22 +17136,22 @@
         <v>31.2</v>
       </c>
       <c r="HL19" s="3" t="n">
-        <v>27.7</v>
+        <v>27.6</v>
       </c>
       <c r="HM19" s="3" t="n">
-        <v>27.7</v>
+        <v>27.6</v>
       </c>
       <c r="HN19" s="3" t="n">
-        <v>23.9</v>
+        <v>23.8</v>
       </c>
       <c r="HO19" s="3" t="n">
-        <v>23.9</v>
+        <v>23.8</v>
       </c>
       <c r="HP19" s="3" t="n">
-        <v>22.1</v>
+        <v>22</v>
       </c>
       <c r="HQ19" s="3" t="n">
-        <v>22.1</v>
+        <v>22</v>
       </c>
       <c r="HR19" s="3" t="n">
         <v>19.7</v>
@@ -17271,13 +17271,13 @@
         <v>7.37</v>
       </c>
       <c r="P20" s="3" t="n">
-        <v>7.15</v>
+        <v>7.16</v>
       </c>
       <c r="Q20" s="3" t="n">
         <v>7.31</v>
       </c>
       <c r="R20" s="3" t="n">
-        <v>1.031</v>
+        <v>1.03</v>
       </c>
       <c r="S20" s="3" t="n">
         <v>7</v>
@@ -17331,10 +17331,10 @@
         <v>45.3</v>
       </c>
       <c r="AH20" s="8" t="n">
-        <v>38.8</v>
+        <v>38.7</v>
       </c>
       <c r="AI20" s="8" t="n">
-        <v>38.3</v>
+        <v>38.2</v>
       </c>
       <c r="AJ20" s="8" t="n">
         <v>32.2</v>
@@ -17376,16 +17376,16 @@
         <v>19.1</v>
       </c>
       <c r="AW20" s="8" t="n">
-        <v>15.3</v>
+        <v>15.2</v>
       </c>
       <c r="AX20" s="8" t="n">
-        <v>15.3</v>
+        <v>15.2</v>
       </c>
       <c r="AY20" s="8" t="n">
         <v>14.4</v>
       </c>
       <c r="AZ20" s="3" t="n">
-        <v>193.07</v>
+        <v>193.06</v>
       </c>
       <c r="BA20" s="4" t="inlineStr">
         <is>
@@ -17874,7 +17874,7 @@
         <v>7.31</v>
       </c>
       <c r="GS20" s="3" t="n">
-        <v>1.78</v>
+        <v>1.79</v>
       </c>
       <c r="GT20" s="3" t="n">
         <v>10.03</v>
@@ -17921,10 +17921,10 @@
         <v>41.8</v>
       </c>
       <c r="HH20" s="3" t="n">
-        <v>35.8</v>
+        <v>35.7</v>
       </c>
       <c r="HI20" s="3" t="n">
-        <v>35.8</v>
+        <v>35.7</v>
       </c>
       <c r="HJ20" s="3" t="n">
         <v>31.2</v>
@@ -17966,10 +17966,10 @@
         <v>19.1</v>
       </c>
       <c r="HW20" s="3" t="n">
-        <v>15.3</v>
+        <v>15.2</v>
       </c>
       <c r="HX20" s="3" t="n">
-        <v>15.3</v>
+        <v>15.2</v>
       </c>
       <c r="HY20" s="3" t="n">
         <v>14.4</v>
@@ -18107,10 +18107,10 @@
         <v>9.1</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>6.79</v>
+        <v>6.8</v>
       </c>
       <c r="L21" s="3" t="n">
-        <v>6.79</v>
+        <v>6.8</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>5.23</v>
@@ -18122,13 +18122,13 @@
         <v>6.22</v>
       </c>
       <c r="P21" s="3" t="n">
-        <v>7.13</v>
+        <v>7.14</v>
       </c>
       <c r="Q21" s="3" t="n">
         <v>6.22</v>
       </c>
       <c r="R21" s="3" t="n">
-        <v>0.872</v>
+        <v>0.871</v>
       </c>
       <c r="S21" s="3" t="n">
         <v>11.8</v>
@@ -18155,22 +18155,22 @@
         </is>
       </c>
       <c r="Y21" s="5" t="n">
-        <v>79.8</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="Z21" s="5" t="n">
         <v>74.09999999999999</v>
       </c>
       <c r="AA21" s="5" t="n">
-        <v>65.59999999999999</v>
+        <v>65.7</v>
       </c>
       <c r="AB21" s="5" t="n">
-        <v>65.09999999999999</v>
+        <v>65.2</v>
       </c>
       <c r="AC21" s="5" t="n">
-        <v>60.4</v>
+        <v>60.6</v>
       </c>
       <c r="AD21" s="5" t="n">
-        <v>59.4</v>
+        <v>59.6</v>
       </c>
       <c r="AE21" s="6" t="n">
         <v>49.5</v>
@@ -18179,19 +18179,19 @@
         <v>49</v>
       </c>
       <c r="AG21" s="7" t="n">
-        <v>45.8</v>
+        <v>45.9</v>
       </c>
       <c r="AH21" s="8" t="n">
-        <v>38.2</v>
+        <v>38.3</v>
       </c>
       <c r="AI21" s="8" t="n">
-        <v>37.7</v>
+        <v>37.8</v>
       </c>
       <c r="AJ21" s="8" t="n">
-        <v>32.5</v>
+        <v>32.6</v>
       </c>
       <c r="AK21" s="8" t="n">
-        <v>31.5</v>
+        <v>31.6</v>
       </c>
       <c r="AL21" s="8" t="n">
         <v>28</v>
@@ -18236,7 +18236,7 @@
         <v>10.8</v>
       </c>
       <c r="AZ21" s="3" t="n">
-        <v>191.73</v>
+        <v>191.9</v>
       </c>
       <c r="BA21" s="4" t="inlineStr">
         <is>
@@ -18245,7 +18245,7 @@
       </c>
       <c r="BB21" s="9" t="inlineStr">
         <is>
-          <t>MORE 5.0 | 59.4% | Edge +1.8</t>
+          <t>MORE 5.0 | 59.6% | Edge +1.8</t>
         </is>
       </c>
       <c r="BC21" s="4" t="inlineStr">
@@ -18257,13 +18257,13 @@
         <v>5</v>
       </c>
       <c r="BE21" s="3" t="n">
-        <v>59.4</v>
+        <v>59.6</v>
       </c>
       <c r="BF21" s="3" t="n">
-        <v>1.79</v>
+        <v>1.8</v>
       </c>
       <c r="BG21" s="3" t="n">
-        <v>18.8</v>
+        <v>19.2</v>
       </c>
       <c r="BH21" s="4" t="inlineStr">
         <is>
@@ -18731,7 +18731,7 @@
         <v>9.59</v>
       </c>
       <c r="GU21" s="3" t="n">
-        <v>15.7</v>
+        <v>15.69</v>
       </c>
       <c r="GV21" s="3" t="n">
         <v>3.92</v>
@@ -18745,22 +18745,22 @@
         </is>
       </c>
       <c r="GY21" s="3" t="n">
-        <v>71.8</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="GZ21" s="3" t="n">
         <v>66.09999999999999</v>
       </c>
       <c r="HA21" s="3" t="n">
-        <v>58.1</v>
+        <v>58.2</v>
       </c>
       <c r="HB21" s="3" t="n">
-        <v>58.1</v>
+        <v>58.2</v>
       </c>
       <c r="HC21" s="3" t="n">
-        <v>54.4</v>
+        <v>54.6</v>
       </c>
       <c r="HD21" s="3" t="n">
-        <v>54.4</v>
+        <v>54.6</v>
       </c>
       <c r="HE21" s="3" t="n">
         <v>45</v>
@@ -18769,19 +18769,19 @@
         <v>45</v>
       </c>
       <c r="HG21" s="3" t="n">
-        <v>42.3</v>
+        <v>42.4</v>
       </c>
       <c r="HH21" s="3" t="n">
-        <v>35.2</v>
+        <v>35.3</v>
       </c>
       <c r="HI21" s="3" t="n">
-        <v>35.2</v>
+        <v>35.3</v>
       </c>
       <c r="HJ21" s="3" t="n">
-        <v>31.5</v>
+        <v>31.6</v>
       </c>
       <c r="HK21" s="3" t="n">
-        <v>31.5</v>
+        <v>31.6</v>
       </c>
       <c r="HL21" s="3" t="n">
         <v>28</v>
@@ -20652,13 +20652,13 @@
         <v>8.970000000000001</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>6.77</v>
+        <v>6.73</v>
       </c>
       <c r="L24" s="3" t="n">
-        <v>6.77</v>
+        <v>6.73</v>
       </c>
       <c r="M24" s="3" t="n">
-        <v>5.23</v>
+        <v>5.21</v>
       </c>
       <c r="N24" s="3" t="n">
         <v>6.34</v>
@@ -20667,13 +20667,13 @@
         <v>6.21</v>
       </c>
       <c r="P24" s="3" t="n">
-        <v>7.15</v>
+        <v>7.09</v>
       </c>
       <c r="Q24" s="3" t="n">
         <v>6.21</v>
       </c>
       <c r="R24" s="3" t="n">
-        <v>0.869</v>
+        <v>0.876</v>
       </c>
       <c r="S24" s="3" t="n">
         <v>10</v>
@@ -20700,88 +20700,88 @@
         </is>
       </c>
       <c r="Y24" s="5" t="n">
-        <v>81.09999999999999</v>
+        <v>81.7</v>
       </c>
       <c r="Z24" s="5" t="n">
-        <v>74.7</v>
+        <v>75</v>
       </c>
       <c r="AA24" s="5" t="n">
-        <v>63.9</v>
+        <v>63.6</v>
       </c>
       <c r="AB24" s="5" t="n">
-        <v>63.4</v>
+        <v>63.1</v>
       </c>
       <c r="AC24" s="5" t="n">
-        <v>59.9</v>
+        <v>59.8</v>
       </c>
       <c r="AD24" s="5" t="n">
-        <v>58.9</v>
+        <v>58.8</v>
       </c>
       <c r="AE24" s="6" t="n">
-        <v>48.6</v>
+        <v>48.3</v>
       </c>
       <c r="AF24" s="7" t="n">
-        <v>48.1</v>
+        <v>47.8</v>
       </c>
       <c r="AG24" s="7" t="n">
-        <v>44.6</v>
+        <v>44.5</v>
       </c>
       <c r="AH24" s="8" t="n">
-        <v>37.8</v>
+        <v>37.7</v>
       </c>
       <c r="AI24" s="8" t="n">
-        <v>37.3</v>
+        <v>37.2</v>
       </c>
       <c r="AJ24" s="8" t="n">
-        <v>31.4</v>
+        <v>31</v>
       </c>
       <c r="AK24" s="8" t="n">
-        <v>30.4</v>
+        <v>30</v>
       </c>
       <c r="AL24" s="8" t="n">
-        <v>27.2</v>
+        <v>26.7</v>
       </c>
       <c r="AM24" s="8" t="n">
-        <v>27.2</v>
+        <v>26.7</v>
       </c>
       <c r="AN24" s="8" t="n">
-        <v>23.1</v>
+        <v>22.7</v>
       </c>
       <c r="AO24" s="8" t="n">
-        <v>21.5</v>
+        <v>20.9</v>
       </c>
       <c r="AP24" s="8" t="n">
-        <v>21.5</v>
+        <v>20.9</v>
       </c>
       <c r="AQ24" s="8" t="n">
-        <v>18.8</v>
+        <v>18.5</v>
       </c>
       <c r="AR24" s="8" t="n">
-        <v>18.8</v>
+        <v>18.5</v>
       </c>
       <c r="AS24" s="8" t="n">
-        <v>17.5</v>
+        <v>17.4</v>
       </c>
       <c r="AT24" s="8" t="n">
-        <v>17.5</v>
+        <v>17.4</v>
       </c>
       <c r="AU24" s="8" t="n">
-        <v>14.2</v>
+        <v>14</v>
       </c>
       <c r="AV24" s="8" t="n">
-        <v>13.2</v>
+        <v>13.1</v>
       </c>
       <c r="AW24" s="8" t="n">
-        <v>13.2</v>
+        <v>13.1</v>
       </c>
       <c r="AX24" s="8" t="n">
-        <v>11.1</v>
+        <v>10.8</v>
       </c>
       <c r="AY24" s="8" t="n">
-        <v>11.1</v>
+        <v>10.8</v>
       </c>
       <c r="AZ24" s="3" t="n">
-        <v>189.21</v>
+        <v>188.58</v>
       </c>
       <c r="BA24" s="4" t="inlineStr">
         <is>
@@ -20790,7 +20790,7 @@
       </c>
       <c r="BB24" s="9" t="inlineStr">
         <is>
-          <t>MORE 5.0 | 58.9% | Edge +1.8</t>
+          <t>MORE 5.0 | 58.8% | Edge +1.7</t>
         </is>
       </c>
       <c r="BC24" s="4" t="inlineStr">
@@ -20802,13 +20802,13 @@
         <v>5</v>
       </c>
       <c r="BE24" s="3" t="n">
-        <v>58.9</v>
+        <v>58.8</v>
       </c>
       <c r="BF24" s="3" t="n">
-        <v>1.77</v>
+        <v>1.73</v>
       </c>
       <c r="BG24" s="3" t="n">
-        <v>17.8</v>
+        <v>17.6</v>
       </c>
       <c r="BH24" s="4" t="inlineStr">
         <is>
@@ -21270,19 +21270,19 @@
         <v>6.21</v>
       </c>
       <c r="GS24" s="3" t="n">
-        <v>0.89</v>
+        <v>0.83</v>
       </c>
       <c r="GT24" s="3" t="n">
-        <v>9.58</v>
+        <v>9.6</v>
       </c>
       <c r="GU24" s="3" t="n">
-        <v>15.66</v>
+        <v>15.73</v>
       </c>
       <c r="GV24" s="3" t="n">
-        <v>3.77</v>
+        <v>3.79</v>
       </c>
       <c r="GW24" s="3" t="n">
-        <v>9.800000000000001</v>
+        <v>9.4</v>
       </c>
       <c r="GX24" s="4" t="inlineStr">
         <is>
@@ -21290,85 +21290,85 @@
         </is>
       </c>
       <c r="GY24" s="3" t="n">
-        <v>73.09999999999999</v>
+        <v>73.7</v>
       </c>
       <c r="GZ24" s="3" t="n">
-        <v>66.7</v>
+        <v>67</v>
       </c>
       <c r="HA24" s="3" t="n">
-        <v>56.4</v>
+        <v>56.1</v>
       </c>
       <c r="HB24" s="3" t="n">
-        <v>56.4</v>
+        <v>56.1</v>
       </c>
       <c r="HC24" s="3" t="n">
-        <v>53.9</v>
+        <v>53.8</v>
       </c>
       <c r="HD24" s="3" t="n">
-        <v>53.9</v>
+        <v>53.8</v>
       </c>
       <c r="HE24" s="3" t="n">
-        <v>44.1</v>
+        <v>43.8</v>
       </c>
       <c r="HF24" s="3" t="n">
-        <v>44.1</v>
+        <v>43.8</v>
       </c>
       <c r="HG24" s="3" t="n">
-        <v>41.1</v>
+        <v>41</v>
       </c>
       <c r="HH24" s="3" t="n">
-        <v>34.8</v>
+        <v>34.7</v>
       </c>
       <c r="HI24" s="3" t="n">
-        <v>34.8</v>
+        <v>34.7</v>
       </c>
       <c r="HJ24" s="3" t="n">
-        <v>30.4</v>
+        <v>30</v>
       </c>
       <c r="HK24" s="3" t="n">
-        <v>30.4</v>
+        <v>30</v>
       </c>
       <c r="HL24" s="3" t="n">
-        <v>27.2</v>
+        <v>26.7</v>
       </c>
       <c r="HM24" s="3" t="n">
-        <v>27.2</v>
+        <v>26.7</v>
       </c>
       <c r="HN24" s="3" t="n">
-        <v>23.1</v>
+        <v>22.7</v>
       </c>
       <c r="HO24" s="3" t="n">
-        <v>21.5</v>
+        <v>20.9</v>
       </c>
       <c r="HP24" s="3" t="n">
-        <v>21.5</v>
+        <v>20.9</v>
       </c>
       <c r="HQ24" s="3" t="n">
-        <v>18.8</v>
+        <v>18.5</v>
       </c>
       <c r="HR24" s="3" t="n">
-        <v>18.8</v>
+        <v>18.5</v>
       </c>
       <c r="HS24" s="3" t="n">
-        <v>17.5</v>
+        <v>17.4</v>
       </c>
       <c r="HT24" s="3" t="n">
-        <v>17.5</v>
+        <v>17.4</v>
       </c>
       <c r="HU24" s="3" t="n">
-        <v>14.2</v>
+        <v>14</v>
       </c>
       <c r="HV24" s="3" t="n">
-        <v>13.2</v>
+        <v>13.1</v>
       </c>
       <c r="HW24" s="3" t="n">
-        <v>13.2</v>
+        <v>13.1</v>
       </c>
       <c r="HX24" s="3" t="n">
-        <v>11.1</v>
+        <v>10.8</v>
       </c>
       <c r="HY24" s="3" t="n">
-        <v>11.1</v>
+        <v>10.8</v>
       </c>
       <c r="HZ24" s="3" t="n">
         <v>8</v>
@@ -22292,13 +22292,13 @@
         <v>8.73</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>6.59</v>
+        <v>6.58</v>
       </c>
       <c r="L26" s="3" t="n">
-        <v>6.59</v>
+        <v>6.58</v>
       </c>
       <c r="M26" s="3" t="n">
-        <v>5.24</v>
+        <v>5.23</v>
       </c>
       <c r="N26" s="3" t="n">
         <v>5.29</v>
@@ -22307,13 +22307,13 @@
         <v>5.56</v>
       </c>
       <c r="P26" s="3" t="n">
-        <v>6.53</v>
+        <v>6.52</v>
       </c>
       <c r="Q26" s="3" t="n">
         <v>5.56</v>
       </c>
       <c r="R26" s="3" t="n">
-        <v>0.851</v>
+        <v>0.853</v>
       </c>
       <c r="S26" s="3" t="n">
         <v>8.4</v>
@@ -22403,10 +22403,10 @@
         <v>15.3</v>
       </c>
       <c r="AT26" s="8" t="n">
-        <v>12</v>
+        <v>11.9</v>
       </c>
       <c r="AU26" s="8" t="n">
-        <v>12</v>
+        <v>11.9</v>
       </c>
       <c r="AV26" s="8" t="n">
         <v>11</v>
@@ -22415,13 +22415,13 @@
         <v>11</v>
       </c>
       <c r="AX26" s="8" t="n">
-        <v>9</v>
+        <v>8.9</v>
       </c>
       <c r="AY26" s="8" t="n">
         <v>7.7</v>
       </c>
       <c r="AZ26" s="3" t="n">
-        <v>185.57</v>
+        <v>185.43</v>
       </c>
       <c r="BA26" s="4" t="inlineStr">
         <is>
@@ -22445,7 +22445,7 @@
         <v>59.2</v>
       </c>
       <c r="BF26" s="3" t="n">
-        <v>1.59</v>
+        <v>1.58</v>
       </c>
       <c r="BG26" s="3" t="n">
         <v>18.4</v>
@@ -22902,13 +22902,13 @@
         <v>5.56</v>
       </c>
       <c r="GS26" s="3" t="n">
-        <v>2.68</v>
+        <v>2.67</v>
       </c>
       <c r="GT26" s="3" t="n">
         <v>8.640000000000001</v>
       </c>
       <c r="GU26" s="3" t="n">
-        <v>14.6</v>
+        <v>14.61</v>
       </c>
       <c r="GV26" s="3" t="n">
         <v>4.42</v>
@@ -22985,10 +22985,10 @@
         <v>15.3</v>
       </c>
       <c r="HT26" s="3" t="n">
-        <v>12</v>
+        <v>11.9</v>
       </c>
       <c r="HU26" s="3" t="n">
-        <v>12</v>
+        <v>11.9</v>
       </c>
       <c r="HV26" s="3" t="n">
         <v>11</v>
@@ -22997,7 +22997,7 @@
         <v>11</v>
       </c>
       <c r="HX26" s="3" t="n">
-        <v>9</v>
+        <v>8.9</v>
       </c>
       <c r="HY26" s="3" t="n">
         <v>7.7</v>
@@ -23135,10 +23135,10 @@
         <v>8.32</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>6.2</v>
+        <v>6.21</v>
       </c>
       <c r="L27" s="3" t="n">
-        <v>6.2</v>
+        <v>6.21</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>4.69</v>
@@ -23156,7 +23156,7 @@
         <v>6.58</v>
       </c>
       <c r="R27" s="3" t="n">
-        <v>1.107</v>
+        <v>1.106</v>
       </c>
       <c r="S27" s="3" t="n">
         <v>1.6</v>
@@ -23198,43 +23198,43 @@
         <v>60</v>
       </c>
       <c r="AD27" s="6" t="n">
-        <v>46.9</v>
+        <v>47</v>
       </c>
       <c r="AE27" s="7" t="n">
-        <v>46.4</v>
+        <v>46.5</v>
       </c>
       <c r="AF27" s="7" t="n">
-        <v>41.4</v>
+        <v>41.5</v>
       </c>
       <c r="AG27" s="7" t="n">
-        <v>40.9</v>
+        <v>41</v>
       </c>
       <c r="AH27" s="8" t="n">
-        <v>33.7</v>
+        <v>33.8</v>
       </c>
       <c r="AI27" s="8" t="n">
-        <v>33.2</v>
+        <v>33.3</v>
       </c>
       <c r="AJ27" s="8" t="n">
-        <v>31.7</v>
+        <v>31.8</v>
       </c>
       <c r="AK27" s="8" t="n">
-        <v>25.9</v>
+        <v>26</v>
       </c>
       <c r="AL27" s="8" t="n">
-        <v>25.9</v>
+        <v>26</v>
       </c>
       <c r="AM27" s="8" t="n">
-        <v>22.6</v>
+        <v>22.7</v>
       </c>
       <c r="AN27" s="8" t="n">
-        <v>22.6</v>
+        <v>22.7</v>
       </c>
       <c r="AO27" s="8" t="n">
-        <v>18.5</v>
+        <v>18.6</v>
       </c>
       <c r="AP27" s="8" t="n">
-        <v>18.5</v>
+        <v>18.6</v>
       </c>
       <c r="AQ27" s="8" t="n">
         <v>16.8</v>
@@ -23243,13 +23243,13 @@
         <v>16.8</v>
       </c>
       <c r="AS27" s="8" t="n">
-        <v>14.5</v>
+        <v>14.6</v>
       </c>
       <c r="AT27" s="8" t="n">
-        <v>14.5</v>
+        <v>14.6</v>
       </c>
       <c r="AU27" s="8" t="n">
-        <v>14.5</v>
+        <v>14.6</v>
       </c>
       <c r="AV27" s="8" t="n">
         <v>13.1</v>
@@ -23264,7 +23264,7 @@
         <v>10.2</v>
       </c>
       <c r="AZ27" s="3" t="n">
-        <v>185.01</v>
+        <v>185.19</v>
       </c>
       <c r="BA27" s="4" t="inlineStr">
         <is>
@@ -23288,7 +23288,7 @@
         <v>60</v>
       </c>
       <c r="BF27" s="3" t="n">
-        <v>1.7</v>
+        <v>1.71</v>
       </c>
       <c r="BG27" s="3" t="n">
         <v>20</v>
@@ -23759,7 +23759,7 @@
         <v>9.119999999999999</v>
       </c>
       <c r="GU27" s="3" t="n">
-        <v>15.76</v>
+        <v>15.75</v>
       </c>
       <c r="GV27" s="3" t="n">
         <v>4.42</v>
@@ -23788,43 +23788,43 @@
         <v>54</v>
       </c>
       <c r="HD27" s="3" t="n">
-        <v>41.9</v>
+        <v>42</v>
       </c>
       <c r="HE27" s="3" t="n">
-        <v>41.9</v>
+        <v>42</v>
       </c>
       <c r="HF27" s="3" t="n">
-        <v>37.4</v>
+        <v>37.5</v>
       </c>
       <c r="HG27" s="3" t="n">
-        <v>37.4</v>
+        <v>37.5</v>
       </c>
       <c r="HH27" s="3" t="n">
-        <v>30.7</v>
+        <v>30.8</v>
       </c>
       <c r="HI27" s="3" t="n">
-        <v>30.7</v>
+        <v>30.8</v>
       </c>
       <c r="HJ27" s="3" t="n">
-        <v>30.7</v>
+        <v>30.8</v>
       </c>
       <c r="HK27" s="3" t="n">
-        <v>25.9</v>
+        <v>26</v>
       </c>
       <c r="HL27" s="3" t="n">
-        <v>25.9</v>
+        <v>26</v>
       </c>
       <c r="HM27" s="3" t="n">
-        <v>22.6</v>
+        <v>22.7</v>
       </c>
       <c r="HN27" s="3" t="n">
-        <v>22.6</v>
+        <v>22.7</v>
       </c>
       <c r="HO27" s="3" t="n">
-        <v>18.5</v>
+        <v>18.6</v>
       </c>
       <c r="HP27" s="3" t="n">
-        <v>18.5</v>
+        <v>18.6</v>
       </c>
       <c r="HQ27" s="3" t="n">
         <v>16.8</v>
@@ -23833,13 +23833,13 @@
         <v>16.8</v>
       </c>
       <c r="HS27" s="3" t="n">
-        <v>14.5</v>
+        <v>14.6</v>
       </c>
       <c r="HT27" s="3" t="n">
-        <v>14.5</v>
+        <v>14.6</v>
       </c>
       <c r="HU27" s="3" t="n">
-        <v>14.5</v>
+        <v>14.6</v>
       </c>
       <c r="HV27" s="3" t="n">
         <v>13.1</v>
@@ -24837,13 +24837,13 @@
         <v>9.27</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>6.51</v>
+        <v>6.52</v>
       </c>
       <c r="L29" s="3" t="n">
-        <v>6.51</v>
+        <v>6.52</v>
       </c>
       <c r="M29" s="3" t="n">
-        <v>5</v>
+        <v>5.01</v>
       </c>
       <c r="N29" s="3" t="n">
         <v>7.83</v>
@@ -24852,13 +24852,13 @@
         <v>7.2</v>
       </c>
       <c r="P29" s="3" t="n">
-        <v>7.22</v>
+        <v>7.23</v>
       </c>
       <c r="Q29" s="3" t="n">
         <v>7.2</v>
       </c>
       <c r="R29" s="3" t="n">
-        <v>0.997</v>
+        <v>0.996</v>
       </c>
       <c r="S29" s="3" t="n">
         <v>12</v>
@@ -24891,22 +24891,22 @@
         <v>71.5</v>
       </c>
       <c r="AA29" s="5" t="n">
-        <v>60.7</v>
+        <v>60.8</v>
       </c>
       <c r="AB29" s="5" t="n">
-        <v>60.2</v>
+        <v>60.3</v>
       </c>
       <c r="AC29" s="6" t="n">
-        <v>56</v>
+        <v>56.1</v>
       </c>
       <c r="AD29" s="7" t="n">
-        <v>55</v>
+        <v>55.1</v>
       </c>
       <c r="AE29" s="7" t="n">
-        <v>45.3</v>
+        <v>45.4</v>
       </c>
       <c r="AF29" s="7" t="n">
-        <v>44.8</v>
+        <v>44.9</v>
       </c>
       <c r="AG29" s="7" t="n">
         <v>41.5</v>
@@ -24918,10 +24918,10 @@
         <v>34.5</v>
       </c>
       <c r="AJ29" s="8" t="n">
-        <v>29.5</v>
+        <v>29.6</v>
       </c>
       <c r="AK29" s="8" t="n">
-        <v>28.5</v>
+        <v>28.6</v>
       </c>
       <c r="AL29" s="8" t="n">
         <v>25.7</v>
@@ -24942,22 +24942,22 @@
         <v>21.1</v>
       </c>
       <c r="AR29" s="8" t="n">
-        <v>19</v>
+        <v>19.1</v>
       </c>
       <c r="AS29" s="8" t="n">
-        <v>19</v>
+        <v>19.1</v>
       </c>
       <c r="AT29" s="8" t="n">
-        <v>18.1</v>
+        <v>18.2</v>
       </c>
       <c r="AU29" s="8" t="n">
-        <v>18.1</v>
+        <v>18.2</v>
       </c>
       <c r="AV29" s="8" t="n">
-        <v>14.7</v>
+        <v>14.8</v>
       </c>
       <c r="AW29" s="8" t="n">
-        <v>14.7</v>
+        <v>14.8</v>
       </c>
       <c r="AX29" s="8" t="n">
         <v>14</v>
@@ -24966,7 +24966,7 @@
         <v>14</v>
       </c>
       <c r="AZ29" s="3" t="n">
-        <v>182.81</v>
+        <v>182.96</v>
       </c>
       <c r="BA29" s="4" t="inlineStr">
         <is>
@@ -24975,7 +24975,7 @@
       </c>
       <c r="BB29" s="9" t="inlineStr">
         <is>
-          <t>MORE 4.0 | 60.2% | Edge +2.5</t>
+          <t>MORE 4.0 | 60.3% | Edge +2.5</t>
         </is>
       </c>
       <c r="BC29" s="4" t="inlineStr">
@@ -24987,13 +24987,13 @@
         <v>4</v>
       </c>
       <c r="BE29" s="3" t="n">
-        <v>60.2</v>
+        <v>60.3</v>
       </c>
       <c r="BF29" s="3" t="n">
-        <v>2.51</v>
+        <v>2.52</v>
       </c>
       <c r="BG29" s="3" t="n">
-        <v>20.4</v>
+        <v>20.6</v>
       </c>
       <c r="BH29" s="4" t="inlineStr">
         <is>
@@ -25455,19 +25455,19 @@
         <v>7.2</v>
       </c>
       <c r="GS29" s="3" t="n">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
       <c r="GT29" s="3" t="n">
-        <v>9.99</v>
+        <v>9.98</v>
       </c>
       <c r="GU29" s="3" t="n">
-        <v>16.97</v>
+        <v>17.95</v>
       </c>
       <c r="GV29" s="3" t="n">
         <v>3.71</v>
       </c>
       <c r="GW29" s="3" t="n">
-        <v>10.5</v>
+        <v>10.6</v>
       </c>
       <c r="GX29" s="4" t="inlineStr">
         <is>
@@ -25481,22 +25481,22 @@
         <v>63.5</v>
       </c>
       <c r="HA29" s="3" t="n">
-        <v>53.2</v>
+        <v>53.3</v>
       </c>
       <c r="HB29" s="3" t="n">
-        <v>53.2</v>
+        <v>53.3</v>
       </c>
       <c r="HC29" s="3" t="n">
-        <v>50</v>
+        <v>50.1</v>
       </c>
       <c r="HD29" s="3" t="n">
-        <v>50</v>
+        <v>50.1</v>
       </c>
       <c r="HE29" s="3" t="n">
-        <v>40.8</v>
+        <v>40.9</v>
       </c>
       <c r="HF29" s="3" t="n">
-        <v>40.8</v>
+        <v>40.9</v>
       </c>
       <c r="HG29" s="3" t="n">
         <v>38</v>
@@ -25508,10 +25508,10 @@
         <v>32</v>
       </c>
       <c r="HJ29" s="3" t="n">
-        <v>28.5</v>
+        <v>28.6</v>
       </c>
       <c r="HK29" s="3" t="n">
-        <v>28.5</v>
+        <v>28.6</v>
       </c>
       <c r="HL29" s="3" t="n">
         <v>25.7</v>
@@ -25532,22 +25532,22 @@
         <v>21.1</v>
       </c>
       <c r="HR29" s="3" t="n">
-        <v>19</v>
+        <v>19.1</v>
       </c>
       <c r="HS29" s="3" t="n">
-        <v>19</v>
+        <v>19.1</v>
       </c>
       <c r="HT29" s="3" t="n">
-        <v>18.1</v>
+        <v>18.2</v>
       </c>
       <c r="HU29" s="3" t="n">
-        <v>18.1</v>
+        <v>18.2</v>
       </c>
       <c r="HV29" s="3" t="n">
-        <v>14.7</v>
+        <v>14.8</v>
       </c>
       <c r="HW29" s="3" t="n">
-        <v>14.7</v>
+        <v>14.8</v>
       </c>
       <c r="HX29" s="3" t="n">
         <v>14</v>
@@ -25703,10 +25703,10 @@
         <v>7.8</v>
       </c>
       <c r="P30" s="3" t="n">
-        <v>5.94</v>
+        <v>5.93</v>
       </c>
       <c r="Q30" s="3" t="n">
-        <v>7.08</v>
+        <v>7.07</v>
       </c>
       <c r="R30" s="3" t="n">
         <v>1.28</v>
@@ -25748,10 +25748,10 @@
         <v>57.3</v>
       </c>
       <c r="AC30" s="7" t="n">
-        <v>44.7</v>
+        <v>44.8</v>
       </c>
       <c r="AD30" s="7" t="n">
-        <v>43.7</v>
+        <v>43.8</v>
       </c>
       <c r="AE30" s="8" t="n">
         <v>39.6</v>
@@ -25793,13 +25793,13 @@
         <v>17.3</v>
       </c>
       <c r="AR30" s="8" t="n">
-        <v>15.8</v>
+        <v>15.7</v>
       </c>
       <c r="AS30" s="8" t="n">
-        <v>15.8</v>
+        <v>15.7</v>
       </c>
       <c r="AT30" s="8" t="n">
-        <v>15.8</v>
+        <v>15.7</v>
       </c>
       <c r="AU30" s="8" t="n">
         <v>13.4</v>
@@ -26295,7 +26295,7 @@
         </is>
       </c>
       <c r="GR30" s="3" t="n">
-        <v>7.08</v>
+        <v>7.07</v>
       </c>
       <c r="GS30" s="3" t="n">
         <v>0</v>
@@ -26330,10 +26330,10 @@
         <v>50.3</v>
       </c>
       <c r="HC30" s="3" t="n">
-        <v>38.7</v>
+        <v>38.8</v>
       </c>
       <c r="HD30" s="3" t="n">
-        <v>38.7</v>
+        <v>38.8</v>
       </c>
       <c r="HE30" s="3" t="n">
         <v>35.1</v>
@@ -26375,13 +26375,13 @@
         <v>17.3</v>
       </c>
       <c r="HR30" s="3" t="n">
-        <v>15.8</v>
+        <v>15.7</v>
       </c>
       <c r="HS30" s="3" t="n">
-        <v>15.8</v>
+        <v>15.7</v>
       </c>
       <c r="HT30" s="3" t="n">
-        <v>15.8</v>
+        <v>15.7</v>
       </c>
       <c r="HU30" s="3" t="n">
         <v>13.4</v>
@@ -26499,168 +26499,168 @@
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Francisco Lindor</t>
+          <t>Jonah Heim</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>NYM</t>
+          <t>ATH</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>ATL</t>
+          <t>TB</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>NYM @ ATL</t>
+          <t>TB @ ATH</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
-          <t>AWAY</t>
+          <t>HOME</t>
         </is>
       </c>
       <c r="I31" s="4" t="inlineStr">
         <is>
-          <t>SS</t>
+          <t>C</t>
         </is>
       </c>
       <c r="J31" s="3" t="n">
-        <v>8.81</v>
+        <v>8.75</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>6.33</v>
+        <v>6.72</v>
       </c>
       <c r="L31" s="3" t="n">
-        <v>6.33</v>
+        <v>6.72</v>
       </c>
       <c r="M31" s="3" t="n">
-        <v>3.89</v>
+        <v>5.2</v>
       </c>
       <c r="N31" s="3" t="n">
-        <v>8.19</v>
+        <v>6.56</v>
       </c>
       <c r="O31" s="3" t="n">
-        <v>7.45</v>
+        <v>6.36</v>
       </c>
       <c r="P31" s="3" t="n">
-        <v>7.29</v>
+        <v>7.2</v>
       </c>
       <c r="Q31" s="3" t="n">
-        <v>7.4</v>
+        <v>6.36</v>
       </c>
       <c r="R31" s="3" t="n">
-        <v>1.021</v>
+        <v>0.883</v>
       </c>
       <c r="S31" s="3" t="n">
-        <v>10.6</v>
+        <v>5.6</v>
       </c>
       <c r="T31" s="3" t="n">
-        <v>9</v>
+        <v>5.2</v>
       </c>
       <c r="U31" s="3" t="n">
-        <v>9.93</v>
+        <v>5.87</v>
       </c>
       <c r="V31" s="4" t="inlineStr">
         <is>
-          <t>11|3|16|21|2</t>
+          <t>7|7|0|7|7</t>
         </is>
       </c>
       <c r="W31" s="4" t="inlineStr">
         <is>
-          <t>11|3|16|21|2|0|5|6|19|7</t>
+          <t>7|7|0|7|7|0|5|0|9|10</t>
         </is>
       </c>
       <c r="X31" s="4" t="inlineStr">
         <is>
-          <t>11|3|16|21|2|0|5|6|19|7|0|4|46|5|4</t>
+          <t>7|7|0|7|7|0|5|0|9|10|20|2|14|0|0</t>
         </is>
       </c>
       <c r="Y31" s="5" t="n">
-        <v>68.59999999999999</v>
+        <v>81.5</v>
       </c>
       <c r="Z31" s="5" t="n">
-        <v>59.4</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="AA31" s="5" t="n">
-        <v>58.9</v>
-      </c>
-      <c r="AB31" s="6" t="n">
-        <v>54.6</v>
-      </c>
-      <c r="AC31" s="7" t="n">
-        <v>53.6</v>
-      </c>
-      <c r="AD31" s="7" t="n">
+        <v>63.8</v>
+      </c>
+      <c r="AB31" s="5" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="AC31" s="5" t="n">
+        <v>59.1</v>
+      </c>
+      <c r="AD31" s="5" t="n">
+        <v>58.1</v>
+      </c>
+      <c r="AE31" s="6" t="n">
+        <v>47.4</v>
+      </c>
+      <c r="AF31" s="7" t="n">
+        <v>46.9</v>
+      </c>
+      <c r="AG31" s="7" t="n">
         <v>43.7</v>
       </c>
-      <c r="AE31" s="7" t="n">
-        <v>43.2</v>
-      </c>
-      <c r="AF31" s="8" t="n">
-        <v>39.9</v>
-      </c>
-      <c r="AG31" s="8" t="n">
-        <v>39.4</v>
-      </c>
       <c r="AH31" s="8" t="n">
-        <v>33.7</v>
+        <v>36.2</v>
       </c>
       <c r="AI31" s="8" t="n">
-        <v>33.2</v>
+        <v>35.7</v>
       </c>
       <c r="AJ31" s="8" t="n">
-        <v>28.3</v>
+        <v>30.5</v>
       </c>
       <c r="AK31" s="8" t="n">
-        <v>27.3</v>
+        <v>29.5</v>
       </c>
       <c r="AL31" s="8" t="n">
-        <v>25</v>
+        <v>26.1</v>
       </c>
       <c r="AM31" s="8" t="n">
-        <v>25</v>
+        <v>26.1</v>
       </c>
       <c r="AN31" s="8" t="n">
-        <v>25</v>
+        <v>22.6</v>
       </c>
       <c r="AO31" s="8" t="n">
-        <v>22.5</v>
+        <v>22.6</v>
       </c>
       <c r="AP31" s="8" t="n">
-        <v>22.5</v>
+        <v>21.1</v>
       </c>
       <c r="AQ31" s="8" t="n">
-        <v>21</v>
+        <v>18.8</v>
       </c>
       <c r="AR31" s="8" t="n">
-        <v>21</v>
+        <v>18.8</v>
       </c>
       <c r="AS31" s="8" t="n">
-        <v>19.3</v>
+        <v>17.8</v>
       </c>
       <c r="AT31" s="8" t="n">
-        <v>19.3</v>
+        <v>17.8</v>
       </c>
       <c r="AU31" s="8" t="n">
-        <v>18.4</v>
+        <v>14.5</v>
       </c>
       <c r="AV31" s="8" t="n">
-        <v>18.4</v>
+        <v>14.5</v>
       </c>
       <c r="AW31" s="8" t="n">
-        <v>14.5</v>
+        <v>13.7</v>
       </c>
       <c r="AX31" s="8" t="n">
-        <v>14.5</v>
+        <v>11</v>
       </c>
       <c r="AY31" s="8" t="n">
-        <v>13.8</v>
+        <v>11</v>
       </c>
       <c r="AZ31" s="3" t="n">
-        <v>182.38</v>
+        <v>182.4</v>
       </c>
       <c r="BA31" s="4" t="inlineStr">
         <is>
@@ -26669,7 +26669,7 @@
       </c>
       <c r="BB31" s="9" t="inlineStr">
         <is>
-          <t>MORE 3.5 | 58.9% | Edge +2.8</t>
+          <t>MORE 5.0 | 58.1% | Edge +1.7</t>
         </is>
       </c>
       <c r="BC31" s="4" t="inlineStr">
@@ -26678,16 +26678,16 @@
         </is>
       </c>
       <c r="BD31" s="3" t="n">
-        <v>3.5</v>
+        <v>5</v>
       </c>
       <c r="BE31" s="3" t="n">
-        <v>58.9</v>
+        <v>58.1</v>
       </c>
       <c r="BF31" s="3" t="n">
-        <v>2.83</v>
+        <v>1.72</v>
       </c>
       <c r="BG31" s="3" t="n">
-        <v>17.8</v>
+        <v>16.2</v>
       </c>
       <c r="BH31" s="4" t="inlineStr">
         <is>
@@ -26695,7 +26695,7 @@
         </is>
       </c>
       <c r="BI31" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BJ31" s="4" t="inlineStr">
         <is>
@@ -26704,24 +26704,24 @@
       </c>
       <c r="BK31" s="4" t="n"/>
       <c r="BL31" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BM31" s="3" t="n">
         <v>7</v>
       </c>
       <c r="BN31" s="4" t="inlineStr">
         <is>
-          <t>2-2-2-1-2-2-2</t>
+          <t>3-3-3-3-4-4-3</t>
         </is>
       </c>
       <c r="BO31" s="3" t="n">
-        <v>85.7</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="BP31" s="3" t="n">
         <v>97</v>
       </c>
       <c r="BQ31" s="3" t="n">
-        <v>4.94</v>
+        <v>4.84</v>
       </c>
       <c r="BR31" s="4" t="inlineStr">
         <is>
@@ -26729,14 +26729,14 @@
         </is>
       </c>
       <c r="BS31" s="3" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="BT31" s="3" t="n">
         <v>1.04</v>
       </c>
       <c r="BU31" s="4" t="inlineStr">
         <is>
-          <t>Bryce Elder</t>
+          <t>Freddy Peralta</t>
         </is>
       </c>
       <c r="BV31" s="4" t="inlineStr">
@@ -26745,124 +26745,124 @@
         </is>
       </c>
       <c r="BW31" s="3" t="n">
-        <v>3.69</v>
+        <v>5.37</v>
       </c>
       <c r="BX31" s="3" t="n">
-        <v>1.2</v>
+        <v>1.52</v>
       </c>
       <c r="BY31" s="3" t="n">
-        <v>0.2079</v>
+        <v>0.2429</v>
       </c>
       <c r="BZ31" s="3" t="n">
-        <v>0.0359</v>
+        <v>0.0358</v>
       </c>
       <c r="CA31" s="3" t="n">
-        <v>0.0794</v>
+        <v>0.09229999999999999</v>
       </c>
       <c r="CB31" s="3" t="n">
-        <v>3.6</v>
+        <v>3.68</v>
       </c>
       <c r="CC31" s="3" t="n">
-        <v>1.24</v>
+        <v>1.14</v>
       </c>
       <c r="CD31" s="3" t="n">
-        <v>0.2025</v>
+        <v>0.2074</v>
       </c>
       <c r="CE31" s="3" t="n">
-        <v>0.0302</v>
+        <v>0.0335</v>
       </c>
       <c r="CF31" s="4" t="inlineStr">
         <is>
-          <t>Truist Park</t>
+          <t>Sutter Health Park</t>
         </is>
       </c>
       <c r="CG31" s="3" t="n">
-        <v>1.01</v>
+        <v>1</v>
       </c>
       <c r="CH31" s="3" t="n">
-        <v>1.03</v>
+        <v>1.055</v>
       </c>
       <c r="CI31" s="3" t="n">
-        <v>88.3</v>
+        <v>100.6</v>
       </c>
       <c r="CJ31" s="3" t="n">
-        <v>5.5</v>
+        <v>7.3</v>
       </c>
       <c r="CK31" s="3" t="n">
-        <v>256</v>
+        <v>225</v>
       </c>
       <c r="CL31" s="3" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="CM31" s="4" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>hot</t>
         </is>
       </c>
       <c r="CN31" s="3" t="n">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="CO31" s="3" t="n">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="CP31" s="3" t="n">
-        <v>0.234</v>
+        <v>0.226</v>
       </c>
       <c r="CQ31" s="3" t="n">
-        <v>0.322</v>
+        <v>0.279</v>
       </c>
       <c r="CR31" s="3" t="n">
-        <v>0.418</v>
+        <v>0.42</v>
       </c>
       <c r="CS31" s="3" t="n">
-        <v>0.74</v>
+        <v>0.699</v>
       </c>
       <c r="CT31" s="3" t="n">
-        <v>193</v>
+        <v>18</v>
       </c>
       <c r="CU31" s="3" t="n">
-        <v>0.745</v>
+        <v>0.611</v>
       </c>
       <c r="CV31" s="3" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="CW31" s="3" t="n">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="CX31" s="3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="CY31" s="3" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="CZ31" s="3" t="n">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="DA31" s="3" t="n">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="DB31" s="3" t="n">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="DC31" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="DD31" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="DE31" s="4" t="inlineStr">
         <is>
-          <t>2026-08-09 @ Pittsburgh Pirates: 11 FS|2026-08-08 @ Pittsburgh Pirates: 3 FS|2026-08-07 @ Pittsburgh Pirates: 16 FS|2026-08-06 @ Cleveland Guardians: 21 FS|2026-08-05 @ Cleveland Guardians: 2 FS</t>
+          <t>2026-08-09 @ Boston Red Sox: 7 FS|2026-08-08 @ Boston Red Sox: 7 FS|2026-08-07 @ Boston Red Sox: 0 FS|2026-08-06 @ Cincinnati Reds: 7 FS|2026-08-05 @ Cincinnati Reds: 7 FS</t>
         </is>
       </c>
       <c r="DF31" s="4" t="inlineStr">
         <is>
-          <t>2026-08-09 @ Pittsburgh Pirates: 11 FS|2026-08-08 @ Pittsburgh Pirates: 3 FS|2026-08-07 @ Pittsburgh Pirates: 16 FS|2026-08-06 @ Cleveland Guardians: 21 FS|2026-08-05 @ Cleveland Guardians: 2 FS|2026-08-04 @ Cleveland Guardians: 0 FS|2026-08-02 vs Miami Marlins: 5 FS|2026-08-01 vs Miami Marlins: 6 FS|2026-07-31 vs Miami Marlins: 19 FS|2026-07-30 vs Miami Marlins: 7 FS</t>
+          <t>2026-08-09 @ Boston Red Sox: 7 FS|2026-08-08 @ Boston Red Sox: 7 FS|2026-08-07 @ Boston Red Sox: 0 FS|2026-08-06 @ Cincinnati Reds: 7 FS|2026-08-05 @ Cincinnati Reds: 7 FS|2026-08-04 @ Cincinnati Reds: 0 FS|2026-08-02 vs Detroit Tigers: 5 FS|2026-08-01 vs Detroit Tigers: 0 FS|2026-07-31 vs Detroit Tigers: 9 FS|2026-07-30 vs Boston Red Sox: 10 FS</t>
         </is>
       </c>
       <c r="DG31" s="4" t="inlineStr">
         <is>
-          <t>2026-08-09 @ Pittsburgh Pirates: 11 FS|2026-08-08 @ Pittsburgh Pirates: 3 FS|2026-08-07 @ Pittsburgh Pirates: 16 FS|2026-08-06 @ Cleveland Guardians: 21 FS|2026-08-05 @ Cleveland Guardians: 2 FS|2026-08-04 @ Cleveland Guardians: 0 FS|2026-08-02 vs Miami Marlins: 5 FS|2026-08-01 vs Miami Marlins: 6 FS|2026-07-31 vs Miami Marlins: 19 FS|2026-07-30 vs Miami Marlins: 7 FS|2026-07-29 vs Atlanta Braves: 0 FS|2026-07-29 vs Atlanta Braves: 4 FS|2026-07-27 vs Atlanta Braves: 46 FS|2026-07-26 vs Los Angeles Dodgers: 5 FS|2026-07-25 vs Los Angeles Dodgers: 4 FS</t>
+          <t>2026-08-09 @ Boston Red Sox: 7 FS|2026-08-08 @ Boston Red Sox: 7 FS|2026-08-07 @ Boston Red Sox: 0 FS|2026-08-06 @ Cincinnati Reds: 7 FS|2026-08-05 @ Cincinnati Reds: 7 FS|2026-08-04 @ Cincinnati Reds: 0 FS|2026-08-02 vs Detroit Tigers: 5 FS|2026-08-01 vs Detroit Tigers: 0 FS|2026-07-31 vs Detroit Tigers: 9 FS|2026-07-30 vs Boston Red Sox: 10 FS|2026-07-29 vs Boston Red Sox: 20 FS|2026-07-28 vs Boston Red Sox: 2 FS|2026-07-27 vs Boston Red Sox: 14 FS|2026-07-26 @ Minnesota Twins: 0 FS|2026-07-25 @ Minnesota Twins: 0 FS</t>
         </is>
       </c>
       <c r="DH31" s="3" t="n">
@@ -26872,10 +26872,10 @@
         <v>30</v>
       </c>
       <c r="DJ31" s="3" t="n">
-        <v>8.27</v>
+        <v>6.03</v>
       </c>
       <c r="DK31" s="3" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="DL31" s="4" t="inlineStr">
         <is>
@@ -26883,13 +26883,13 @@
         </is>
       </c>
       <c r="DM31" s="3" t="n">
-        <v>8.289999999999999</v>
+        <v>4.71</v>
       </c>
       <c r="DN31" s="3" t="n">
-        <v>10.36</v>
+        <v>6.29</v>
       </c>
       <c r="DO31" s="3" t="n">
-        <v>0.268</v>
+        <v>0.222</v>
       </c>
       <c r="DP31" s="4" t="inlineStr">
         <is>
@@ -26897,40 +26897,40 @@
         </is>
       </c>
       <c r="DQ31" s="3" t="n">
-        <v>8.27</v>
+        <v>6.03</v>
       </c>
       <c r="DR31" s="3" t="n">
-        <v>2.266</v>
+        <v>1.517</v>
       </c>
       <c r="DS31" s="3" t="n">
-        <v>0.2344</v>
+        <v>0.2069</v>
       </c>
       <c r="DT31" s="3" t="n">
-        <v>0.09379999999999999</v>
+        <v>0.1034</v>
       </c>
       <c r="DU31" s="3" t="n">
-        <v>0.0625</v>
+        <v>0.0345</v>
       </c>
       <c r="DV31" s="3" t="n">
-        <v>0.1094</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="DW31" s="3" t="n">
-        <v>0.0156</v>
+        <v>0</v>
       </c>
       <c r="DX31" s="3" t="n">
-        <v>8.69</v>
+        <v>8.970000000000001</v>
       </c>
       <c r="DY31" s="3" t="n">
-        <v>9.26</v>
+        <v>8.41</v>
       </c>
       <c r="DZ31" s="3" t="n">
-        <v>9.710000000000001</v>
+        <v>8.75</v>
       </c>
       <c r="EA31" s="3" t="n">
-        <v>8.720000000000001</v>
+        <v>8.49</v>
       </c>
       <c r="EB31" s="3" t="n">
-        <v>7.78</v>
+        <v>8.91</v>
       </c>
       <c r="EC31" s="3" t="n">
         <v>28</v>
@@ -26948,25 +26948,25 @@
         <v>20</v>
       </c>
       <c r="EH31" s="3" t="n">
-        <v>218</v>
+        <v>239</v>
       </c>
       <c r="EI31" s="3" t="n">
-        <v>84.87</v>
+        <v>82.76000000000001</v>
       </c>
       <c r="EJ31" s="3" t="n">
-        <v>32.11</v>
+        <v>23.01</v>
       </c>
       <c r="EK31" s="3" t="n">
-        <v>1.83</v>
+        <v>2.09</v>
       </c>
       <c r="EL31" s="3" t="n">
-        <v>29.36</v>
+        <v>29.71</v>
       </c>
       <c r="EM31" s="3" t="n">
-        <v>0.394</v>
+        <v>0.358</v>
       </c>
       <c r="EN31" s="3" t="n">
-        <v>0.9689</v>
+        <v>0.8913</v>
       </c>
       <c r="EO31" s="3" t="n">
         <v>1</v>
@@ -26978,10 +26978,10 @@
         <v>1</v>
       </c>
       <c r="ER31" s="3" t="n">
-        <v>1.0629</v>
+        <v>0.9895</v>
       </c>
       <c r="ES31" s="3" t="n">
-        <v>549</v>
+        <v>448</v>
       </c>
       <c r="ET31" s="4" t="inlineStr">
         <is>
@@ -26989,10 +26989,10 @@
         </is>
       </c>
       <c r="EU31" s="3" t="n">
-        <v>1.0059</v>
+        <v>1.0841</v>
       </c>
       <c r="EV31" s="3" t="n">
-        <v>46</v>
+        <v>13</v>
       </c>
       <c r="EW31" s="4" t="inlineStr">
         <is>
@@ -27000,52 +27000,52 @@
         </is>
       </c>
       <c r="EX31" s="3" t="n">
-        <v>218</v>
+        <v>239</v>
       </c>
       <c r="EY31" s="3" t="n">
-        <v>84.87</v>
+        <v>82.76000000000001</v>
       </c>
       <c r="EZ31" s="3" t="n">
         <v>12</v>
       </c>
       <c r="FA31" s="3" t="n">
-        <v>21.03</v>
+        <v>18.32</v>
       </c>
       <c r="FB31" s="3" t="n">
-        <v>32.44</v>
+        <v>35</v>
       </c>
       <c r="FC31" s="3" t="n">
-        <v>14.7</v>
+        <v>13</v>
       </c>
       <c r="FD31" s="3" t="n">
-        <v>65.59999999999999</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="FE31" s="3" t="n">
-        <v>19.7</v>
+        <v>20.9</v>
       </c>
       <c r="FF31" s="3" t="n">
-        <v>1.0195</v>
+        <v>1.0512</v>
       </c>
       <c r="FG31" s="3" t="n">
-        <v>1.0053</v>
+        <v>0.9984</v>
       </c>
       <c r="FH31" s="3" t="n">
-        <v>1.0392</v>
+        <v>1.0451</v>
       </c>
       <c r="FI31" s="3" t="n">
-        <v>1.0105</v>
+        <v>0.9968</v>
       </c>
       <c r="FJ31" s="3" t="n">
-        <v>1.0553</v>
+        <v>1.0401</v>
       </c>
       <c r="FK31" s="3" t="n">
-        <v>1.011</v>
+        <v>0.9954</v>
       </c>
       <c r="FL31" s="3" t="n">
-        <v>9.18</v>
+        <v>5.65</v>
       </c>
       <c r="FM31" s="3" t="n">
-        <v>0.91</v>
+        <v>-0.38</v>
       </c>
       <c r="FN31" s="4" t="inlineStr">
         <is>
@@ -27090,7 +27090,7 @@
         <v>27</v>
       </c>
       <c r="FZ31" s="3" t="n">
-        <v>1.1061</v>
+        <v>0.8625</v>
       </c>
       <c r="GA31" s="3" t="n">
         <v>27</v>
@@ -27099,43 +27099,43 @@
         <v>1</v>
       </c>
       <c r="GC31" s="3" t="n">
-        <v>0.1209</v>
+        <v>0.1358</v>
       </c>
       <c r="GD31" s="3" t="n">
-        <v>0.0355</v>
+        <v>0.0542</v>
       </c>
       <c r="GE31" s="3" t="n">
-        <v>0.0058</v>
+        <v>0.0031</v>
       </c>
       <c r="GF31" s="3" t="n">
-        <v>0.0433</v>
+        <v>0.0364</v>
       </c>
       <c r="GG31" s="3" t="n">
-        <v>0.0927</v>
+        <v>0.0761</v>
       </c>
       <c r="GH31" s="3" t="n">
-        <v>0.0117</v>
+        <v>0.01</v>
       </c>
       <c r="GI31" s="3" t="n">
-        <v>0.2012</v>
+        <v>0.2053</v>
       </c>
       <c r="GJ31" s="3" t="n">
-        <v>0.3301</v>
+        <v>0.4737</v>
       </c>
       <c r="GK31" s="3" t="n">
-        <v>0.38</v>
+        <v>0.307</v>
       </c>
       <c r="GL31" s="3" t="n">
-        <v>0.2899</v>
+        <v>0.2193</v>
       </c>
       <c r="GM31" s="3" t="n">
-        <v>0.1244</v>
+        <v>0.1181</v>
       </c>
       <c r="GN31" s="3" t="n">
-        <v>0.1199</v>
+        <v>0.1464</v>
       </c>
       <c r="GO31" s="3" t="n">
-        <v>0.0132</v>
+        <v>0.0081</v>
       </c>
       <c r="GP31" s="3" t="n">
         <v>1</v>
@@ -27146,22 +27146,22 @@
         </is>
       </c>
       <c r="GR31" s="3" t="n">
-        <v>7.4</v>
+        <v>6.36</v>
       </c>
       <c r="GS31" s="3" t="n">
-        <v>0</v>
+        <v>0.78</v>
       </c>
       <c r="GT31" s="3" t="n">
-        <v>9</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="GU31" s="3" t="n">
-        <v>17.17</v>
+        <v>15.8</v>
       </c>
       <c r="GV31" s="3" t="n">
-        <v>3.85</v>
+        <v>3.97</v>
       </c>
       <c r="GW31" s="3" t="n">
-        <v>11.3</v>
+        <v>7.7</v>
       </c>
       <c r="GX31" s="4" t="inlineStr">
         <is>
@@ -27169,85 +27169,85 @@
         </is>
       </c>
       <c r="GY31" s="3" t="n">
-        <v>60.6</v>
+        <v>73.5</v>
       </c>
       <c r="GZ31" s="3" t="n">
-        <v>51.4</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="HA31" s="3" t="n">
-        <v>51.4</v>
+        <v>56.3</v>
       </c>
       <c r="HB31" s="3" t="n">
-        <v>47.6</v>
+        <v>56.3</v>
       </c>
       <c r="HC31" s="3" t="n">
-        <v>47.6</v>
+        <v>53.1</v>
       </c>
       <c r="HD31" s="3" t="n">
-        <v>38.7</v>
+        <v>53.1</v>
       </c>
       <c r="HE31" s="3" t="n">
-        <v>38.7</v>
+        <v>42.9</v>
       </c>
       <c r="HF31" s="3" t="n">
-        <v>35.9</v>
+        <v>42.9</v>
       </c>
       <c r="HG31" s="3" t="n">
-        <v>35.9</v>
+        <v>40.2</v>
       </c>
       <c r="HH31" s="3" t="n">
-        <v>30.7</v>
+        <v>33.2</v>
       </c>
       <c r="HI31" s="3" t="n">
-        <v>30.7</v>
+        <v>33.2</v>
       </c>
       <c r="HJ31" s="3" t="n">
-        <v>27.3</v>
+        <v>29.5</v>
       </c>
       <c r="HK31" s="3" t="n">
-        <v>27.3</v>
+        <v>29.5</v>
       </c>
       <c r="HL31" s="3" t="n">
-        <v>25</v>
+        <v>26.1</v>
       </c>
       <c r="HM31" s="3" t="n">
-        <v>25</v>
+        <v>26.1</v>
       </c>
       <c r="HN31" s="3" t="n">
-        <v>25</v>
+        <v>22.6</v>
       </c>
       <c r="HO31" s="3" t="n">
-        <v>22.5</v>
+        <v>22.6</v>
       </c>
       <c r="HP31" s="3" t="n">
-        <v>22.5</v>
+        <v>21.1</v>
       </c>
       <c r="HQ31" s="3" t="n">
-        <v>21</v>
+        <v>18.8</v>
       </c>
       <c r="HR31" s="3" t="n">
-        <v>21</v>
+        <v>18.8</v>
       </c>
       <c r="HS31" s="3" t="n">
-        <v>19.3</v>
+        <v>17.8</v>
       </c>
       <c r="HT31" s="3" t="n">
-        <v>19.3</v>
+        <v>17.8</v>
       </c>
       <c r="HU31" s="3" t="n">
-        <v>18.4</v>
+        <v>14.5</v>
       </c>
       <c r="HV31" s="3" t="n">
-        <v>18.4</v>
+        <v>14.5</v>
       </c>
       <c r="HW31" s="3" t="n">
-        <v>14.5</v>
+        <v>13.7</v>
       </c>
       <c r="HX31" s="3" t="n">
-        <v>14.5</v>
+        <v>11</v>
       </c>
       <c r="HY31" s="3" t="n">
-        <v>13.8</v>
+        <v>11</v>
       </c>
       <c r="HZ31" s="3" t="n">
         <v>8</v>

</xml_diff>